<commit_message>
Update berita 2026-08-04 19:16 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-05.xlsx
+++ b/data/berita_antara_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -477,33 +477,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>video</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
+          <t>Pelatihan warga binaan Lapas Kupang hasilkan barang bernilai ekonomi</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
+          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
+          <t>ANTARA - Lembaga Pemasyarakatan Kelas IIA Kupang, Nusa Tenggara Timur, pada Senin (3/8), terus mengoptimalkan pembinaan kemandirian warga binaan melalui berbagai program pemberdayaan, mulai dari pelatihan keterampilan, pendidikan, hingga ketahanan pangan. Program ini diharapkan menjadi bekal bagi warga binaan setelah bebas sekaligus meningkatkan nilai ekonomi hasil karya mereka. (Johannes Viandinando/Denno Ramdha Asmara/Winanto)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
+          <t>https://www.antaranews.com/berita/5679020/pelatihan-warga-binaan-lapas-kupang-hasilkan-barang-bernilai-ekonomi</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PELATIHAN-WARGA-BINAAN-LAPAS-KUPANG-HASILKAN-BARANG-BERNILAI-EKONOMI.jpg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -515,33 +515,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>video</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>Pemkot Ambon wajibkan ASN registrasi digitalisasi Bansos</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
+          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
+          <t>ANTARA - Pemerintah Kota (Pemkot) Ambon melakukan registrasi digitalisasi Bantuan Sosial (Bansos) di Pattimura Park, kota Ambon, Maluku, Selasa (4/8). Kegiatan digitalisasi bansos ini diwajibkan untuk seluruh Apartur Sipil Negara di lingkup Pemkot Ambon. (Alfian Sanusi/Denno Ramdha Asmara/Winanto)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5678964/pemkot-ambon-wajibkan-asn-registrasi-digitalisasi-bansos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKOT-AMBON-WAJIBKAN-ASN-REGISTRASI-DIGITALISASI-BANSOS.jpg</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -558,28 +558,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
+          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
+          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
+          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
+          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -596,28 +596,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
+          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
+          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -634,28 +634,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
+          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
+          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
+          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -667,33 +667,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -705,33 +705,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
+          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
+          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
+          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -743,33 +743,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
+          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
+          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -781,33 +781,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
+          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
+          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -819,33 +819,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
+          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
+          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
+          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -857,33 +857,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
+          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -895,33 +895,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
+          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
+          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
+          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -933,33 +933,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
+          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -971,33 +971,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
+          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1009,33 +1009,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
+          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
+          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
+          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1047,33 +1047,33 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
+          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
+          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
+          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1085,33 +1085,33 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
+          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
+          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
+          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1128,28 +1128,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
+          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1166,28 +1166,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
+          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1204,28 +1204,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
+          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1242,28 +1242,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
+          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
+          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1280,28 +1280,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
+          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1318,28 +1318,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1356,28 +1356,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1394,28 +1394,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1432,28 +1432,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1470,28 +1470,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1508,28 +1508,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1546,28 +1546,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1584,990 +1584,1446 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
+          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
           <t>ANTARA - Presiden RI Prabowo Subianto mengantar langsung kepulangan Perdana Menteri Thailand Anutin Charnvirakul dari Lanud Halim Perdanakusuma, Jakarta, Selasa (4/8). Kepulangan PM Anutin menutup rangkaian kunjungannya di Indonesia selama dua hari yang memperkuat kemitraan strategis kedua negara di sektor keamanan, ekonomi, hingga energi.
 (Cahya Sari/Irfansyah Naufal Nasution/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679719/presiden-prabowo-antar-langsung-kepulangan-pm-thailand-dari-halim</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-192451.jpg</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
         <is>
           <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
         <is>
           <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
         <is>
           <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
         <is>
           <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
         <is>
           <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
         <is>
           <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
         <is>
           <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
         <is>
           <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
         <is>
           <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
         <is>
           <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
         <is>
           <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
         <is>
           <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
         <is>
           <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
         <is>
           <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
         <is>
           <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
         <is>
           <t>ANTARA - Dewan Harian Daerah (DHD) Badan Pembudayaan Kejuangan 45 Sumatera Utara resmi dilantik dan disaksikan langsung oleh Gubernur Sumatera Utara Bobby Nasution di Kantor Gubernur Sumut, Selasa, (4/8). Bobby menyebutkan tujuan dilantiknya DHD 45 Sumut ini untuk meneruskan semangat juang para pahlawan terdahulu agar tetap diterapkan hingga saat ini.
 (M. Valery Maulidzar S/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679368/pelantikan-dhd-45-gubernur-sumut-tekankan-semangat-juang-pahlawan</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PELANTIKAN-DHD-45-GUBERNUR-SUMUT-TEKANKAN-SEMANGAT-JUANG-PAHLAWAN.jpg</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t>Kabut tebal hentikan lalu lintas maritim di Selat Bosporus Turki</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
         <is>
           <t>ANTARA - Lalu lintas maritim di Selat Bosporus Istanbul, Turki, dihentikan pada Senin (2/8) karena kabut tebal.Kabut tebal juga mengganggu layanan feri antara sisi Eropa dan Asia Istanbul, dengan feri penumpang dan kendaraan yang dihentikan hingga pemberitahuan lebih lanjut. (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679345/kabut-tebal-hentikan-lalu-lintas-maritim-di-selat-bosporus-turki</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-161506.jpg</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>Mendag targetkan neraca dagang pada Juli 2026 kembali surplus</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Perdagangan Budi Santoso menargetkan neraca perdagangan Indonesia akan kembali mencetak surplus pada Juli 2026. Mendag di Jakarta pada Selasa (4/8) menyebut hal itu diproyeksikan seiring mulai stabilnya harga minyak dunia. (Sanya Dinda Susanti/Pradanna Putra Tampi/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679321/mendag-targetkan-neraca-dagang-pada-juli-2026-kembali-surplus</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-160042.jpg</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
         <is>
           <t>TNI tembus medan ekstrem selama 12 hari antarkan bantuan ke Puncak</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
         <is>
           <t>ANTARA - Komando Operasi TNI Habema berhasil menyalurkan dua ton bantuan kemanusiaan kepada masyarakat di Distrik Agandugume, Oneri, dan Lambewi, Kabupaten Puncak, Papua Tengah. Bantuan tersebut tiba setelah personel TNI berjalan kaki  selama 12 hari melintasi pegunungan dengan medan ekstrem dan cuaca yang tidak menentu. (Laksa Mahendra/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679297/tni-tembus-medan-ekstrem-selama-12-hari-antarkan-bantuan-ke-puncak</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_TNI-TEMBUS-MEDAN-EKSTREM-SELAMA-12-HARI-ANTARKAN-BANTUAN-KE-PUNCAK.jpg</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>Menko Zulhas bantah isu Kopdes penyebab tutupnya warung kelontong</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Koordinator Bidang Pangan, Zulkifli Hasan, membantah isu yang menyebut kehadiran Koperasi Desa/Kelurahan Merah Putih akan menyebabkan penutupan warung kelontong. Zulhas menegaskan Koperasi Merah Putih merupakan infrastruktur pemerintah yang dibentuk untuk memperkuat penyaluran berbagai subsidi dan bantuan kepada masyarakat. (Shintia Aryanti Krisna/Dudy Yanuwardhana/Winanto)</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679253/menko-zulhas-bantah-isu-kopdes-penyebab-tutupnya-warung-kelontong</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/MENKO-ZULHAS-BANTAH-ISU-KOPDES.jpg</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>Pemkot Yogyakarta berikan vaksin HPV perdana pada anak laki-laki</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
         <is>
           <t>ANTARA -Dinas Kesehatan Kota Yogyakarta memperluas sasaran program Vaksinasi Human Papillomavirus (HPV) yang tidak hanya diperuntukan bagi anak perempuan, namun juga menyasar anak laki-laki usia 11 tahun. Pemberian vaksin HPV tersebut dilakukan perdana di Sekolah Dasar Intis School Kotagede pada Selasa (4/8).(Imam Prasetyo Nugroho/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679247/pemkot-yogyakarta-berikan-vaksin-hpv-perdana-pada-anak-laki-laki</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-154404.jpg</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
         <is>
           <t>Pemerintah targetkan perdagangan RI-Thailand tembus 20 miliar dolar AS</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Perdagangan Budi Santoso usai menghadiri Indonesia-Thailand Business Forum, di Jakarta, Selasa (4/8), menyatakan, pemerintah menargetkan nilai perdagangan Indonesia dan Thailand meningkat menjadi lebih dari 20 miliar dolar AS dari posisi saat ini sebesar 17,7 miliar dolar AS. Target tersebut akan diupayakan melalui peningkatan pertemuan bilateral untuk mengurangi hambatan perdagangan dan memperluas akses pasar kedua negara. (Nabila Athifa/Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Winanto)</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679237/pemerintah-targetkan-perdagangan-ri-thailand-tembus-20-miliar-dolar-as</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TARGETKAN-PERDAGANGAN-RI-THAILAND-TEMBUS-20-MILIAR-DOLAR-AS.jpg</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
         <is>
           <t>Pemkab Banjarnegara fasilitasi warga deteksi dini kesehatan mata</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
         <is>
           <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, bersama Yayasan Satu Karsa Karya (YSKK) meluncurkan program penguatan sistem dan pelayanan kesehatan mata yang efektif dan inklusif. Kegiatan ini  merupakan upaya untuk mencegah gangguan penglihatan dan katarak dengan penanganan terintegrasi dari tingkat pelayanan primer hingga sekunder melalui penjaringan keluhan pada berbagai kelembagaan yang dekat dengan masyarakat. (Addin Alfath Amajida/Dudy Yanuwardhana/Winanto)</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679229/pemkab-banjarnegara-fasilitasi-warga-deteksi-dini-kesehatan-mata</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKAB-BANJARNEGARA-FASILITASI-WARGA.jpg</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
         <is>
           <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa (4/8), yang dihadiri Perdana Menteri (PM) Thailand Anutin Charnvirakul. Dalam kesempatan tersebut ditandatangani sejumlah perjanjian kerja sama di bidang perekonomian. (Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>Dilanda cuaca panas, nakes Lhokseumawe bagikan masker untuk cegah ISPA</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
         <is>
           <t>ANTARA - Dilanda cuaca panas hingga 35 derajat celcius, tim nakes dari Puskesmas Mon Gedong, Kecamatan Banda Sakti, Kota Lhokseumawe, Aceh, membagikan masker bagi pengendara di Simpang Empat Masjid Islamic Center, sebagai salah satu upaya pencegahan penyakit Infeksi Saluran Pernapasan Akut (ISPA), Selasa (4/8). (Try Vanny S/Denno Ramdha Asmara/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679057/dilanda-cuaca-panas-nakes-lhokseumawe-bagikan-masker-untuk-cegah-ispa</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G68" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/DILANDA-CUACA-PANAS-NAKES-LHOKSEUMAWE-BAGIKAN-MASKER-UNTUK-CEGAH-ISPA.jpg</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Pelatihan warga binaan Lapas Kupang hasilkan barang bernilai ekonomi</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>ANTARA - Lembaga Pemasyarakatan Kelas IIA Kupang, Nusa Tenggara Timur, pada Senin (3/8), terus mengoptimalkan pembinaan kemandirian warga binaan melalui berbagai program pemberdayaan, mulai dari pelatihan keterampilan, pendidikan, hingga ketahanan pangan. Program ini diharapkan menjadi bekal bagi warga binaan setelah bebas sekaligus meningkatkan nilai ekonomi hasil karya mereka. (Johannes Viandinando/Denno Ramdha Asmara/Winanto)</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679020/pelatihan-warga-binaan-lapas-kupang-hasilkan-barang-bernilai-ekonomi</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PELATIHAN-WARGA-BINAAN-LAPAS-KUPANG-HASILKAN-BARANG-BERNILAI-EKONOMI.jpg</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Pemkot Ambon wajibkan ASN registrasi digitalisasi Bansos</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 00:25:01 +0700</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah Kota (Pemkot) Ambon melakukan registrasi digitalisasi Bantuan Sosial (Bansos) di Pattimura Park, kota Ambon, Maluku, Selasa (4/8). Kegiatan digitalisasi bansos ini diwajibkan untuk seluruh Apartur Sipil Negara di lingkup Pemkot Ambon. (Alfian Sanusi/Denno Ramdha Asmara/Winanto)</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5678964/pemkot-ambon-wajibkan-asn-registrasi-digitalisasi-bansos</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKOT-AMBON-WAJIBKAN-ASN-REGISTRASI-DIGITALISASI-BANSOS.jpg</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
+      <c r="H68" t="inlineStr">
         <is>
           <t>antara</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-04 21:00 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-05.xlsx
+++ b/data/berita_antara_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -558,28 +558,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
+          <t>Potret gelombang panas dan karhutla di Eropa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
+          <t>Wed, 05 Aug 2026 03:29:29 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
+          <t>Eropa sedang menghadapi gelombang panas berkepanjangan dan kekeringan yang meluas. Kondisi tersebut semakin menambah ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
+          <t>https://www.antaranews.com/berita/5680159/potret-gelombang-panas-dan-karhutla-di-eropa</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000022_20260804_CBMFN0A001.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -596,28 +596,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
+          <t>Bluebird bukukan pendapatan Rp2,97 triliun di Semester I 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
+          <t>Wed, 05 Aug 2026 03:02:51 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
+          <t>PT Blue Bird Tbk (Bird) membukukan pendapatan sebesar Rp2,97 triliun pada Semester I 2026, didukung kinerja seluruh ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
+          <t>https://www.antaranews.com/berita/5680157/bluebird-bukukan-pendapatan-rp297-triliun-di-semester-i-2026</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/B0EE512C-6D50-4F78-AADA-5319D04B8721.jpeg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -634,28 +634,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
+          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
+          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
+          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
+          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -672,28 +672,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
+          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
+          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -710,28 +710,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
+          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
+          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
+          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -748,28 +748,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
+          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
+          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
+          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -786,28 +786,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
+          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
+          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
+          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
+          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -824,28 +824,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
+          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
+          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
+          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -862,28 +862,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
+          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
+          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
+          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
+          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -900,28 +900,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
+          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
+          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
+          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
+          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -938,28 +938,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
+          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
+          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -976,28 +976,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
+          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
+          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1014,28 +1014,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
+          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
+          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
+          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
+          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1052,28 +1052,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
+          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
+          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1090,28 +1090,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
+          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
+          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
+          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
+          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1123,33 +1123,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
+          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
+          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1161,33 +1161,33 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1204,28 +1204,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
+          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1242,28 +1242,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
+          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1280,28 +1280,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
+          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1318,28 +1318,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
+          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
+          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1356,28 +1356,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
+          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
+          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1394,28 +1394,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
+          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
+          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1432,28 +1432,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
+          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
+          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
+          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1470,28 +1470,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
+          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1508,28 +1508,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
+          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
+          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1546,28 +1546,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
+          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
+          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1584,28 +1584,28 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
+          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
+          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1622,28 +1622,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
+          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
+          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
+          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1660,28 +1660,28 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
+          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
+          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1698,28 +1698,28 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
+          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
+          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1736,28 +1736,28 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
+          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
+          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1774,28 +1774,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
+          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
+          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
+          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1812,28 +1812,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
+          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1850,28 +1850,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1888,28 +1888,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1926,28 +1926,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1964,28 +1964,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2002,28 +2002,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2040,28 +2040,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2078,28 +2078,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2116,105 +2116,105 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
+          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
           <t>ANTARA - Presiden RI Prabowo Subianto mengantar langsung kepulangan Perdana Menteri Thailand Anutin Charnvirakul dari Lanud Halim Perdanakusuma, Jakarta, Selasa (4/8). Kepulangan PM Anutin menutup rangkaian kunjungannya di Indonesia selama dua hari yang memperkuat kemitraan strategis kedua negara di sektor keamanan, ekonomi, hingga energi.
 (Cahya Sari/Irfansyah Naufal Nasution/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679719/presiden-prabowo-antar-langsung-kepulangan-pm-thailand-dari-halim</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-192451.jpg</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2231,28 +2231,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
+          <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
+          <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2269,28 +2269,28 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
+          <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
+          <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
+          <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2307,28 +2307,28 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
+          <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
+          <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2345,28 +2345,28 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
+          <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
+          <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
+          <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2383,28 +2383,28 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
+          <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
+          <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
+          <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2421,28 +2421,28 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
+          <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
+          <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2459,28 +2459,28 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
+          <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
+          <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2497,28 +2497,28 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
+          <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
+          <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2535,28 +2535,28 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
+          <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
+          <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2573,28 +2573,28 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
+          <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
+          <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2611,28 +2611,28 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
+          <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
+          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
+          <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2649,105 +2649,105 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
+          <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
+          <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
           <t>ANTARA - Dewan Harian Daerah (DHD) Badan Pembudayaan Kejuangan 45 Sumatera Utara resmi dilantik dan disaksikan langsung oleh Gubernur Sumatera Utara Bobby Nasution di Kantor Gubernur Sumut, Selasa, (4/8). Bobby menyebutkan tujuan dilantiknya DHD 45 Sumut ini untuk meneruskan semangat juang para pahlawan terdahulu agar tetap diterapkan hingga saat ini.
 (M. Valery Maulidzar S/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679368/pelantikan-dhd-45-gubernur-sumut-tekankan-semangat-juang-pahlawan</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PELANTIKAN-DHD-45-GUBERNUR-SUMUT-TEKANKAN-SEMANGAT-JUANG-PAHLAWAN.jpg</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Kabut tebal hentikan lalu lintas maritim di Selat Bosporus Turki</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>ANTARA - Lalu lintas maritim di Selat Bosporus Istanbul, Turki, dihentikan pada Senin (2/8) karena kabut tebal.Kabut tebal juga mengganggu layanan feri antara sisi Eropa dan Asia Istanbul, dengan feri penumpang dan kendaraan yang dihentikan hingga pemberitahuan lebih lanjut. (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679345/kabut-tebal-hentikan-lalu-lintas-maritim-di-selat-bosporus-turki</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-161506.jpg</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Mendag targetkan neraca dagang pada Juli 2026 kembali surplus</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>ANTARA - Menteri Perdagangan Budi Santoso menargetkan neraca perdagangan Indonesia akan kembali mencetak surplus pada Juli 2026. Mendag di Jakarta pada Selasa (4/8) menyebut hal itu diproyeksikan seiring mulai stabilnya harga minyak dunia. (Sanya Dinda Susanti/Pradanna Putra Tampi/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679321/mendag-targetkan-neraca-dagang-pada-juli-2026-kembali-surplus</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-160042.jpg</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2764,28 +2764,28 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TNI tembus medan ekstrem selama 12 hari antarkan bantuan ke Puncak</t>
+          <t>Kabut tebal hentikan lalu lintas maritim di Selat Bosporus Turki</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ANTARA - Komando Operasi TNI Habema berhasil menyalurkan dua ton bantuan kemanusiaan kepada masyarakat di Distrik Agandugume, Oneri, dan Lambewi, Kabupaten Puncak, Papua Tengah. Bantuan tersebut tiba setelah personel TNI berjalan kaki  selama 12 hari melintasi pegunungan dengan medan ekstrem dan cuaca yang tidak menentu. (Laksa Mahendra/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Lalu lintas maritim di Selat Bosporus Istanbul, Turki, dihentikan pada Senin (2/8) karena kabut tebal.Kabut tebal juga mengganggu layanan feri antara sisi Eropa dan Asia Istanbul, dengan feri penumpang dan kendaraan yang dihentikan hingga pemberitahuan lebih lanjut. (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679297/tni-tembus-medan-ekstrem-selama-12-hari-antarkan-bantuan-ke-puncak</t>
+          <t>https://www.antaranews.com/berita/5679345/kabut-tebal-hentikan-lalu-lintas-maritim-di-selat-bosporus-turki</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_TNI-TEMBUS-MEDAN-EKSTREM-SELAMA-12-HARI-ANTARKAN-BANTUAN-KE-PUNCAK.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-161506.jpg</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -2802,28 +2802,28 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Menko Zulhas bantah isu Kopdes penyebab tutupnya warung kelontong</t>
+          <t>Mendag targetkan neraca dagang pada Juli 2026 kembali surplus</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Koordinator Bidang Pangan, Zulkifli Hasan, membantah isu yang menyebut kehadiran Koperasi Desa/Kelurahan Merah Putih akan menyebabkan penutupan warung kelontong. Zulhas menegaskan Koperasi Merah Putih merupakan infrastruktur pemerintah yang dibentuk untuk memperkuat penyaluran berbagai subsidi dan bantuan kepada masyarakat. (Shintia Aryanti Krisna/Dudy Yanuwardhana/Winanto)</t>
+          <t>ANTARA - Menteri Perdagangan Budi Santoso menargetkan neraca perdagangan Indonesia akan kembali mencetak surplus pada Juli 2026. Mendag di Jakarta pada Selasa (4/8) menyebut hal itu diproyeksikan seiring mulai stabilnya harga minyak dunia. (Sanya Dinda Susanti/Pradanna Putra Tampi/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679253/menko-zulhas-bantah-isu-kopdes-penyebab-tutupnya-warung-kelontong</t>
+          <t>https://www.antaranews.com/berita/5679321/mendag-targetkan-neraca-dagang-pada-juli-2026-kembali-surplus</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/MENKO-ZULHAS-BANTAH-ISU-KOPDES.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-160042.jpg</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2840,28 +2840,28 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Pemkot Yogyakarta berikan vaksin HPV perdana pada anak laki-laki</t>
+          <t>TNI tembus medan ekstrem selama 12 hari antarkan bantuan ke Puncak</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ANTARA -Dinas Kesehatan Kota Yogyakarta memperluas sasaran program Vaksinasi Human Papillomavirus (HPV) yang tidak hanya diperuntukan bagi anak perempuan, namun juga menyasar anak laki-laki usia 11 tahun. Pemberian vaksin HPV tersebut dilakukan perdana di Sekolah Dasar Intis School Kotagede pada Selasa (4/8).(Imam Prasetyo Nugroho/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Komando Operasi TNI Habema berhasil menyalurkan dua ton bantuan kemanusiaan kepada masyarakat di Distrik Agandugume, Oneri, dan Lambewi, Kabupaten Puncak, Papua Tengah. Bantuan tersebut tiba setelah personel TNI berjalan kaki  selama 12 hari melintasi pegunungan dengan medan ekstrem dan cuaca yang tidak menentu. (Laksa Mahendra/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679247/pemkot-yogyakarta-berikan-vaksin-hpv-perdana-pada-anak-laki-laki</t>
+          <t>https://www.antaranews.com/berita/5679297/tni-tembus-medan-ekstrem-selama-12-hari-antarkan-bantuan-ke-puncak</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-154404.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_TNI-TEMBUS-MEDAN-EKSTREM-SELAMA-12-HARI-ANTARKAN-BANTUAN-KE-PUNCAK.jpg</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2878,28 +2878,28 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Pemerintah targetkan perdagangan RI-Thailand tembus 20 miliar dolar AS</t>
+          <t>Menko Zulhas bantah isu Kopdes penyebab tutupnya warung kelontong</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Perdagangan Budi Santoso usai menghadiri Indonesia-Thailand Business Forum, di Jakarta, Selasa (4/8), menyatakan, pemerintah menargetkan nilai perdagangan Indonesia dan Thailand meningkat menjadi lebih dari 20 miliar dolar AS dari posisi saat ini sebesar 17,7 miliar dolar AS. Target tersebut akan diupayakan melalui peningkatan pertemuan bilateral untuk mengurangi hambatan perdagangan dan memperluas akses pasar kedua negara. (Nabila Athifa/Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Winanto)</t>
+          <t>ANTARA - Menteri Koordinator Bidang Pangan, Zulkifli Hasan, membantah isu yang menyebut kehadiran Koperasi Desa/Kelurahan Merah Putih akan menyebabkan penutupan warung kelontong. Zulhas menegaskan Koperasi Merah Putih merupakan infrastruktur pemerintah yang dibentuk untuk memperkuat penyaluran berbagai subsidi dan bantuan kepada masyarakat. (Shintia Aryanti Krisna/Dudy Yanuwardhana/Winanto)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679237/pemerintah-targetkan-perdagangan-ri-thailand-tembus-20-miliar-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5679253/menko-zulhas-bantah-isu-kopdes-penyebab-tutupnya-warung-kelontong</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TARGETKAN-PERDAGANGAN-RI-THAILAND-TEMBUS-20-MILIAR-DOLAR-AS.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/MENKO-ZULHAS-BANTAH-ISU-KOPDES.jpg</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2916,28 +2916,28 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Pemkab Banjarnegara fasilitasi warga deteksi dini kesehatan mata</t>
+          <t>Pemkot Yogyakarta berikan vaksin HPV perdana pada anak laki-laki</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, bersama Yayasan Satu Karsa Karya (YSKK) meluncurkan program penguatan sistem dan pelayanan kesehatan mata yang efektif dan inklusif. Kegiatan ini  merupakan upaya untuk mencegah gangguan penglihatan dan katarak dengan penanganan terintegrasi dari tingkat pelayanan primer hingga sekunder melalui penjaringan keluhan pada berbagai kelembagaan yang dekat dengan masyarakat. (Addin Alfath Amajida/Dudy Yanuwardhana/Winanto)</t>
+          <t>ANTARA -Dinas Kesehatan Kota Yogyakarta memperluas sasaran program Vaksinasi Human Papillomavirus (HPV) yang tidak hanya diperuntukan bagi anak perempuan, namun juga menyasar anak laki-laki usia 11 tahun. Pemberian vaksin HPV tersebut dilakukan perdana di Sekolah Dasar Intis School Kotagede pada Selasa (4/8).(Imam Prasetyo Nugroho/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679229/pemkab-banjarnegara-fasilitasi-warga-deteksi-dini-kesehatan-mata</t>
+          <t>https://www.antaranews.com/berita/5679247/pemkot-yogyakarta-berikan-vaksin-hpv-perdana-pada-anak-laki-laki</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKAB-BANJARNEGARA-FASILITASI-WARGA.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-154404.jpg</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2954,28 +2954,28 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
+          <t>Pemerintah targetkan perdagangan RI-Thailand tembus 20 miliar dolar AS</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa (4/8), yang dihadiri Perdana Menteri (PM) Thailand Anutin Charnvirakul. Dalam kesempatan tersebut ditandatangani sejumlah perjanjian kerja sama di bidang perekonomian. (Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Menteri Perdagangan Budi Santoso usai menghadiri Indonesia-Thailand Business Forum, di Jakarta, Selasa (4/8), menyatakan, pemerintah menargetkan nilai perdagangan Indonesia dan Thailand meningkat menjadi lebih dari 20 miliar dolar AS dari posisi saat ini sebesar 17,7 miliar dolar AS. Target tersebut akan diupayakan melalui peningkatan pertemuan bilateral untuk mengurangi hambatan perdagangan dan memperluas akses pasar kedua negara. (Nabila Athifa/Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Winanto)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
+          <t>https://www.antaranews.com/berita/5679237/pemerintah-targetkan-perdagangan-ri-thailand-tembus-20-miliar-dolar-as</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TARGETKAN-PERDAGANGAN-RI-THAILAND-TEMBUS-20-MILIAR-DOLAR-AS.jpg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2992,38 +2992,114 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Dilanda cuaca panas, nakes Lhokseumawe bagikan masker untuk cegah ISPA</t>
+          <t>Pemkab Banjarnegara fasilitasi warga deteksi dini kesehatan mata</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:15:01 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
+          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, bersama Yayasan Satu Karsa Karya (YSKK) meluncurkan program penguatan sistem dan pelayanan kesehatan mata yang efektif dan inklusif. Kegiatan ini  merupakan upaya untuk mencegah gangguan penglihatan dan katarak dengan penanganan terintegrasi dari tingkat pelayanan primer hingga sekunder melalui penjaringan keluhan pada berbagai kelembagaan yang dekat dengan masyarakat. (Addin Alfath Amajida/Dudy Yanuwardhana/Winanto)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679229/pemkab-banjarnegara-fasilitasi-warga-deteksi-dini-kesehatan-mata</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKAB-BANJARNEGARA-FASILITASI-WARGA.jpg</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa (4/8), yang dihadiri Perdana Menteri (PM) Thailand Anutin Charnvirakul. Dalam kesempatan tersebut ditandatangani sejumlah perjanjian kerja sama di bidang perekonomian. (Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Dilanda cuaca panas, nakes Lhokseumawe bagikan masker untuk cegah ISPA</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
           <t>ANTARA - Dilanda cuaca panas hingga 35 derajat celcius, tim nakes dari Puskesmas Mon Gedong, Kecamatan Banda Sakti, Kota Lhokseumawe, Aceh, membagikan masker bagi pengendara di Simpang Empat Masjid Islamic Center, sebagai salah satu upaya pencegahan penyakit Infeksi Saluran Pernapasan Akut (ISPA), Selasa (4/8). (Try Vanny S/Denno Ramdha Asmara/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679057/dilanda-cuaca-panas-nakes-lhokseumawe-bagikan-masker-untuk-cegah-ispa</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/DILANDA-CUACA-PANAS-NAKES-LHOKSEUMAWE-BAGIKAN-MASKER-UNTUK-CEGAH-ISPA.jpg</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>antara</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H68"/>
+  <autoFilter ref="A1:H70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-04 22:12 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-05.xlsx
+++ b/data/berita_antara_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,10 +419,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -553,33 +553,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>video</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Potret gelombang panas dan karhutla di Eropa</t>
+          <t>Dilanda cuaca panas, nakes Lhokseumawe bagikan masker untuk cegah ISPA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 03:29:29 +0700</t>
+          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Eropa sedang menghadapi gelombang panas berkepanjangan dan kekeringan yang meluas. Kondisi tersebut semakin menambah ...</t>
+          <t>ANTARA - Dilanda cuaca panas hingga 35 derajat celcius, tim nakes dari Puskesmas Mon Gedong, Kecamatan Banda Sakti, Kota Lhokseumawe, Aceh, membagikan masker bagi pengendara di Simpang Empat Masjid Islamic Center, sebagai salah satu upaya pencegahan penyakit Infeksi Saluran Pernapasan Akut (ISPA), Selasa (4/8). (Try Vanny S/Denno Ramdha Asmara/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680159/potret-gelombang-panas-dan-karhutla-di-eropa</t>
+          <t>https://www.antaranews.com/berita/5679057/dilanda-cuaca-panas-nakes-lhokseumawe-bagikan-masker-untuk-cegah-ispa</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000022_20260804_CBMFN0A001.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/DILANDA-CUACA-PANAS-NAKES-LHOKSEUMAWE-BAGIKAN-MASKER-UNTUK-CEGAH-ISPA.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -596,28 +596,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bluebird bukukan pendapatan Rp2,97 triliun di Semester I 2026</t>
+          <t>Kemarin, surpres penggantian Kapolri hingga harga BBM subsidi tak naik</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 03:02:51 +0700</t>
+          <t>Wed, 05 Aug 2026 04:58:19 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PT Blue Bird Tbk (Bird) membukukan pendapatan sebesar Rp2,97 triliun pada Semester I 2026, didukung kinerja seluruh ...</t>
+          <t>Berbagai kabar politik telah diwartakan Kantor Berita ANTARA pada Selasa (4/8), mulai dari Komisi III membantah adanya ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680157/bluebird-bukukan-pendapatan-rp297-triliun-di-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5680176/kemarin-surpres-penggantian-kapolri-hingga-harga-bbm-subsidi-tak-naik</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/B0EE512C-6D50-4F78-AADA-5319D04B8721.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1001272341_1.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -634,28 +634,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
+          <t>Kabag Keuangan DPRD Ponorogo tersangka korupsi tunjangan perumahan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
+          <t>Wed, 05 Aug 2026 04:35:14 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
+          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo, menetapkan Kepala Bagian (Kabag) Keuangan sekretariat DPRD setempat ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
+          <t>https://www.antaranews.com/video/5679951/kabag-keuangan-dprd-ponorogo-tersangka-korupsi-tunjangan-perumahan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_23_53_24.Still477.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -672,28 +672,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
+          <t>Kemarin, Febrie ajukan praperadilan hingga nasib status jaksanya</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
+          <t>Wed, 05 Aug 2026 04:28:47 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
+          <t>Berbagai kabar hukum telah diwartakan Kantor Berita ANTARA pada Selasa (4/8), mulai dari mantan Jampidsus Febrie ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
+          <t>https://www.antaranews.com/berita/5680172/kemarin-febrie-ajukan-praperadilan-hingga-nasib-status-jaksanya</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087202.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -705,33 +705,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
+          <t>Jetour bakal hadirkan lebih banyak pilihan NEV ke pasar Indonesia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
+          <t>Wed, 05 Aug 2026 04:24:54 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
+          <t>Jenama mobil listrik asal China, Jetour bakal hadirkan lebih banyak pilihan kendaraan energi baru (NEV) ke pasar . ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
+          <t>https://otomotif.antaranews.com/berita/5680169/jetour-bakal-hadirkan-lebih-banyak-pilihan-nev-ke-pasar-indonesia</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/WhatsApp-Image-2026-05-27-at-17.54.18.jpeg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -748,28 +748,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
+          <t>OJK bantah alami defisit anggaran dalam laporan keuangan 2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
+          <t>Wed, 05 Aug 2026 04:16:57 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
+          <t>Wakil Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Hernawan Bekti Sasongko membantah adanya isu defisit ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
+          <t>https://www.antaranews.com/berita/5680167/ojk-bantah-alami-defisit-anggaran-dalam-laporan-keuangan-2025</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/31b157c6-a45a-436b-8256-05aff0c845e7.jpeg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -786,28 +786,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
+          <t>Gempa M 5,6 guncang barat laut Halmahera Barat, tak berpotensi tsunami</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
+          <t>Wed, 05 Aug 2026 04:04:11 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) melaporkan gempa dengan magnitudo 5,6 mengguncang barat laut ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
+          <t>https://www.antaranews.com/berita/5680163/gempa-m-56-guncang-barat-laut-halmahera-barat-tak-berpotensi-tsunami</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/ilustrasi-gempa-3.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -824,28 +824,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
+          <t>Potret gelombang panas dan karhutla di Eropa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
+          <t>Wed, 05 Aug 2026 03:29:29 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
+          <t>Eropa sedang menghadapi gelombang panas berkepanjangan dan kekeringan yang meluas. Kondisi tersebut semakin menambah ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
+          <t>https://www.antaranews.com/berita/5680159/potret-gelombang-panas-dan-karhutla-di-eropa</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000022_20260804_CBMFN0A001.jpg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -862,28 +862,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
+          <t>Bluebird bukukan pendapatan Rp2,97 triliun di Semester I 2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
+          <t>Wed, 05 Aug 2026 03:02:51 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
+          <t>PT Blue Bird Tbk (Bird) membukukan pendapatan sebesar Rp2,97 triliun pada Semester I 2026, didukung kinerja seluruh ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
+          <t>https://www.antaranews.com/berita/5680157/bluebird-bukukan-pendapatan-rp297-triliun-di-semester-i-2026</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/B0EE512C-6D50-4F78-AADA-5319D04B8721.jpeg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -900,28 +900,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
+          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
+          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
+          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
+          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -938,28 +938,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
+          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
+          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -976,28 +976,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
+          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
+          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
+          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1014,28 +1014,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
+          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
+          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
+          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1052,28 +1052,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
+          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
+          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1090,28 +1090,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
+          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
+          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
+          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1128,28 +1128,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
+          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
+          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
+          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
+          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1166,28 +1166,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
+          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
+          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
+          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
+          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1199,33 +1199,33 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
+          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1237,33 +1237,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1275,33 +1275,33 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
+          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
+          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1313,33 +1313,33 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
+          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1351,33 +1351,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
+          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
+          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1389,33 +1389,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
+          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
+          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1427,33 +1427,33 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
+          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
+          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
+          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1470,28 +1470,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
+          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1508,28 +1508,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
+          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1546,28 +1546,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1584,28 +1584,28 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
+          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
+          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1622,28 +1622,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
+          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
+          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1660,28 +1660,28 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
+          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
+          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1698,28 +1698,28 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
+          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
+          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
+          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1736,28 +1736,28 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
+          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
+          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1774,28 +1774,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
+          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
+          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1812,28 +1812,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
+          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
+          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1850,28 +1850,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
+          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
+          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
+          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1888,28 +1888,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
+          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1926,28 +1926,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1964,28 +1964,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2002,28 +2002,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2040,28 +2040,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+          <t>Kabag Keuangan DPRD Ponorogo tersangka korupsi tunjangan perumahan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo, menetapkan Kepala Bagian (Kabag) Keuangan sekretariat DPRD setempat sebagai tersangka dalam kasus dugaan korupsi tunjangan perumahan anggota DPRD setempat, yang merugikan negara hingga 3,6 miliar rupiah. (Rindhu Dwi Kartiko/Arif Prada/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+          <t>https://www.antaranews.com/berita/5679951/kabag-keuangan-dprd-ponorogo-tersangka-korupsi-tunjangan-perumahan</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_23_53_24.Still477.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2078,28 +2078,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2116,28 +2116,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2154,28 +2154,28 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2192,333 +2192,333 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
+          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
           <t>ANTARA - Presiden RI Prabowo Subianto mengantar langsung kepulangan Perdana Menteri Thailand Anutin Charnvirakul dari Lanud Halim Perdanakusuma, Jakarta, Selasa (4/8). Kepulangan PM Anutin menutup rangkaian kunjungannya di Indonesia selama dua hari yang memperkuat kemitraan strategis kedua negara di sektor keamanan, ekonomi, hingga energi.
 (Cahya Sari/Irfansyah Naufal Nasution/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679719/presiden-prabowo-antar-langsung-kepulangan-pm-thailand-dari-halim</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-192451.jpg</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2535,28 +2535,28 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
+          <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
+          <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2573,28 +2573,28 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
+          <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
+          <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2611,28 +2611,28 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
+          <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
+          <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2649,28 +2649,28 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
+          <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
+          <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2687,28 +2687,28 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
+          <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
+          <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
+          <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2725,333 +2725,333 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
+          <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
+          <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
           <t>ANTARA - Dewan Harian Daerah (DHD) Badan Pembudayaan Kejuangan 45 Sumatera Utara resmi dilantik dan disaksikan langsung oleh Gubernur Sumatera Utara Bobby Nasution di Kantor Gubernur Sumut, Selasa, (4/8). Bobby menyebutkan tujuan dilantiknya DHD 45 Sumut ini untuk meneruskan semangat juang para pahlawan terdahulu agar tetap diterapkan hingga saat ini.
 (M. Valery Maulidzar S/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679368/pelantikan-dhd-45-gubernur-sumut-tekankan-semangat-juang-pahlawan</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PELANTIKAN-DHD-45-GUBERNUR-SUMUT-TEKANKAN-SEMANGAT-JUANG-PAHLAWAN.jpg</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Kabut tebal hentikan lalu lintas maritim di Selat Bosporus Turki</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>ANTARA - Lalu lintas maritim di Selat Bosporus Istanbul, Turki, dihentikan pada Senin (2/8) karena kabut tebal.Kabut tebal juga mengganggu layanan feri antara sisi Eropa dan Asia Istanbul, dengan feri penumpang dan kendaraan yang dihentikan hingga pemberitahuan lebih lanjut. (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679345/kabut-tebal-hentikan-lalu-lintas-maritim-di-selat-bosporus-turki</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-161506.jpg</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Mendag targetkan neraca dagang pada Juli 2026 kembali surplus</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>ANTARA - Menteri Perdagangan Budi Santoso menargetkan neraca perdagangan Indonesia akan kembali mencetak surplus pada Juli 2026. Mendag di Jakarta pada Selasa (4/8) menyebut hal itu diproyeksikan seiring mulai stabilnya harga minyak dunia. (Sanya Dinda Susanti/Pradanna Putra Tampi/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679321/mendag-targetkan-neraca-dagang-pada-juli-2026-kembali-surplus</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-160042.jpg</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>TNI tembus medan ekstrem selama 12 hari antarkan bantuan ke Puncak</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>ANTARA - Komando Operasi TNI Habema berhasil menyalurkan dua ton bantuan kemanusiaan kepada masyarakat di Distrik Agandugume, Oneri, dan Lambewi, Kabupaten Puncak, Papua Tengah. Bantuan tersebut tiba setelah personel TNI berjalan kaki  selama 12 hari melintasi pegunungan dengan medan ekstrem dan cuaca yang tidak menentu. (Laksa Mahendra/Andi Bagasela/Roy Rosa Bachtiar)</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679297/tni-tembus-medan-ekstrem-selama-12-hari-antarkan-bantuan-ke-puncak</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_TNI-TEMBUS-MEDAN-EKSTREM-SELAMA-12-HARI-ANTARKAN-BANTUAN-KE-PUNCAK.jpg</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Menko Zulhas bantah isu Kopdes penyebab tutupnya warung kelontong</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>ANTARA - Menteri Koordinator Bidang Pangan, Zulkifli Hasan, membantah isu yang menyebut kehadiran Koperasi Desa/Kelurahan Merah Putih akan menyebabkan penutupan warung kelontong. Zulhas menegaskan Koperasi Merah Putih merupakan infrastruktur pemerintah yang dibentuk untuk memperkuat penyaluran berbagai subsidi dan bantuan kepada masyarakat. (Shintia Aryanti Krisna/Dudy Yanuwardhana/Winanto)</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679253/menko-zulhas-bantah-isu-kopdes-penyebab-tutupnya-warung-kelontong</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/MENKO-ZULHAS-BANTAH-ISU-KOPDES.jpg</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Pemkot Yogyakarta berikan vaksin HPV perdana pada anak laki-laki</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>ANTARA -Dinas Kesehatan Kota Yogyakarta memperluas sasaran program Vaksinasi Human Papillomavirus (HPV) yang tidak hanya diperuntukan bagi anak perempuan, namun juga menyasar anak laki-laki usia 11 tahun. Pemberian vaksin HPV tersebut dilakukan perdana di Sekolah Dasar Intis School Kotagede pada Selasa (4/8).(Imam Prasetyo Nugroho/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679247/pemkot-yogyakarta-berikan-vaksin-hpv-perdana-pada-anak-laki-laki</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-154404.jpg</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Pemerintah targetkan perdagangan RI-Thailand tembus 20 miliar dolar AS</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>ANTARA - Menteri Perdagangan Budi Santoso usai menghadiri Indonesia-Thailand Business Forum, di Jakarta, Selasa (4/8), menyatakan, pemerintah menargetkan nilai perdagangan Indonesia dan Thailand meningkat menjadi lebih dari 20 miliar dolar AS dari posisi saat ini sebesar 17,7 miliar dolar AS. Target tersebut akan diupayakan melalui peningkatan pertemuan bilateral untuk mengurangi hambatan perdagangan dan memperluas akses pasar kedua negara. (Nabila Athifa/Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Winanto)</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679237/pemerintah-targetkan-perdagangan-ri-thailand-tembus-20-miliar-dolar-as</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TARGETKAN-PERDAGANGAN-RI-THAILAND-TEMBUS-20-MILIAR-DOLAR-AS.jpg</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Pemkab Banjarnegara fasilitasi warga deteksi dini kesehatan mata</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, bersama Yayasan Satu Karsa Karya (YSKK) meluncurkan program penguatan sistem dan pelayanan kesehatan mata yang efektif dan inklusif. Kegiatan ini  merupakan upaya untuk mencegah gangguan penglihatan dan katarak dengan penanganan terintegrasi dari tingkat pelayanan primer hingga sekunder melalui penjaringan keluhan pada berbagai kelembagaan yang dekat dengan masyarakat. (Addin Alfath Amajida/Dudy Yanuwardhana/Winanto)</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679229/pemkab-banjarnegara-fasilitasi-warga-deteksi-dini-kesehatan-mata</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKAB-BANJARNEGARA-FASILITASI-WARGA.jpg</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa (4/8), yang dihadiri Perdana Menteri (PM) Thailand Anutin Charnvirakul. Dalam kesempatan tersebut ditandatangani sejumlah perjanjian kerja sama di bidang perekonomian. (Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Roy Rosa Bachtiar)</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3068,28 +3068,28 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dilanda cuaca panas, nakes Lhokseumawe bagikan masker untuk cegah ISPA</t>
+          <t>Kabut tebal hentikan lalu lintas maritim di Selat Bosporus Turki</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:00:01 +0700</t>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ANTARA - Dilanda cuaca panas hingga 35 derajat celcius, tim nakes dari Puskesmas Mon Gedong, Kecamatan Banda Sakti, Kota Lhokseumawe, Aceh, membagikan masker bagi pengendara di Simpang Empat Masjid Islamic Center, sebagai salah satu upaya pencegahan penyakit Infeksi Saluran Pernapasan Akut (ISPA), Selasa (4/8). (Try Vanny S/Denno Ramdha Asmara/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Lalu lintas maritim di Selat Bosporus Istanbul, Turki, dihentikan pada Senin (2/8) karena kabut tebal.Kabut tebal juga mengganggu layanan feri antara sisi Eropa dan Asia Istanbul, dengan feri penumpang dan kendaraan yang dihentikan hingga pemberitahuan lebih lanjut. (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679057/dilanda-cuaca-panas-nakes-lhokseumawe-bagikan-masker-untuk-cegah-ispa</t>
+          <t>https://www.antaranews.com/berita/5679345/kabut-tebal-hentikan-lalu-lintas-maritim-di-selat-bosporus-turki</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/DILANDA-CUACA-PANAS-NAKES-LHOKSEUMAWE-BAGIKAN-MASKER-UNTUK-CEGAH-ISPA.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-161506.jpg</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3098,8 +3098,274 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Mendag targetkan neraca dagang pada Juli 2026 kembali surplus</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Perdagangan Budi Santoso menargetkan neraca perdagangan Indonesia akan kembali mencetak surplus pada Juli 2026. Mendag di Jakarta pada Selasa (4/8) menyebut hal itu diproyeksikan seiring mulai stabilnya harga minyak dunia. (Sanya Dinda Susanti/Pradanna Putra Tampi/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679321/mendag-targetkan-neraca-dagang-pada-juli-2026-kembali-surplus</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-160042.jpg</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>TNI tembus medan ekstrem selama 12 hari antarkan bantuan ke Puncak</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ANTARA - Komando Operasi TNI Habema berhasil menyalurkan dua ton bantuan kemanusiaan kepada masyarakat di Distrik Agandugume, Oneri, dan Lambewi, Kabupaten Puncak, Papua Tengah. Bantuan tersebut tiba setelah personel TNI berjalan kaki  selama 12 hari melintasi pegunungan dengan medan ekstrem dan cuaca yang tidak menentu. (Laksa Mahendra/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679297/tni-tembus-medan-ekstrem-selama-12-hari-antarkan-bantuan-ke-puncak</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_TNI-TEMBUS-MEDAN-EKSTREM-SELAMA-12-HARI-ANTARKAN-BANTUAN-KE-PUNCAK.jpg</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Menko Zulhas bantah isu Kopdes penyebab tutupnya warung kelontong</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Koordinator Bidang Pangan, Zulkifli Hasan, membantah isu yang menyebut kehadiran Koperasi Desa/Kelurahan Merah Putih akan menyebabkan penutupan warung kelontong. Zulhas menegaskan Koperasi Merah Putih merupakan infrastruktur pemerintah yang dibentuk untuk memperkuat penyaluran berbagai subsidi dan bantuan kepada masyarakat. (Shintia Aryanti Krisna/Dudy Yanuwardhana/Winanto)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679253/menko-zulhas-bantah-isu-kopdes-penyebab-tutupnya-warung-kelontong</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/MENKO-ZULHAS-BANTAH-ISU-KOPDES.jpg</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pemkot Yogyakarta berikan vaksin HPV perdana pada anak laki-laki</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ANTARA -Dinas Kesehatan Kota Yogyakarta memperluas sasaran program Vaksinasi Human Papillomavirus (HPV) yang tidak hanya diperuntukan bagi anak perempuan, namun juga menyasar anak laki-laki usia 11 tahun. Pemberian vaksin HPV tersebut dilakukan perdana di Sekolah Dasar Intis School Kotagede pada Selasa (4/8).(Imam Prasetyo Nugroho/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679247/pemkot-yogyakarta-berikan-vaksin-hpv-perdana-pada-anak-laki-laki</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-154404.jpg</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Pemerintah targetkan perdagangan RI-Thailand tembus 20 miliar dolar AS</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Perdagangan Budi Santoso usai menghadiri Indonesia-Thailand Business Forum, di Jakarta, Selasa (4/8), menyatakan, pemerintah menargetkan nilai perdagangan Indonesia dan Thailand meningkat menjadi lebih dari 20 miliar dolar AS dari posisi saat ini sebesar 17,7 miliar dolar AS. Target tersebut akan diupayakan melalui peningkatan pertemuan bilateral untuk mengurangi hambatan perdagangan dan memperluas akses pasar kedua negara. (Nabila Athifa/Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Winanto)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679237/pemerintah-targetkan-perdagangan-ri-thailand-tembus-20-miliar-dolar-as</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TARGETKAN-PERDAGANGAN-RI-THAILAND-TEMBUS-20-MILIAR-DOLAR-AS.jpg</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Pemkab Banjarnegara fasilitasi warga deteksi dini kesehatan mata</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, bersama Yayasan Satu Karsa Karya (YSKK) meluncurkan program penguatan sistem dan pelayanan kesehatan mata yang efektif dan inklusif. Kegiatan ini  merupakan upaya untuk mencegah gangguan penglihatan dan katarak dengan penanganan terintegrasi dari tingkat pelayanan primer hingga sekunder melalui penjaringan keluhan pada berbagai kelembagaan yang dekat dengan masyarakat. (Addin Alfath Amajida/Dudy Yanuwardhana/Winanto)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679229/pemkab-banjarnegara-fasilitasi-warga-deteksi-dini-kesehatan-mata</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKAB-BANJARNEGARA-FASILITASI-WARGA.jpg</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa (4/8), yang dihadiri Perdana Menteri (PM) Thailand Anutin Charnvirakul. Dalam kesempatan tersebut ditandatangani sejumlah perjanjian kerja sama di bidang perekonomian. (Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H70"/>
+  <autoFilter ref="A1:H77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-04 23:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-05.xlsx
+++ b/data/berita_antara_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -596,28 +596,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kemarin, surpres penggantian Kapolri hingga harga BBM subsidi tak naik</t>
+          <t>DKI kemarin, pajak kendaraan listrik hingga TJ turunkan penumpang</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:58:19 +0700</t>
+          <t>Wed, 05 Aug 2026 06:49:19 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Berbagai kabar politik telah diwartakan Kantor Berita ANTARA pada Selasa (4/8), mulai dari Komisi III membantah adanya ...</t>
+          <t>Anggota Badan Pembentukan Peraturan Daerah (Bapemperda) DPRD DKI Jakarta, Yusuf mengusulkan penerapan pajak terhadap ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680176/kemarin-surpres-penggantian-kapolri-hingga-harga-bbm-subsidi-tak-naik</t>
+          <t>https://www.antaranews.com/berita/5680195/dki-kemarin-pajak-kendaraan-listrik-hingga-tj-turunkan-penumpang</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1001272341_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/08/IMG_20251008_190653.jpg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -634,28 +634,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kabag Keuangan DPRD Ponorogo tersangka korupsi tunjangan perumahan</t>
+          <t>Humaniora kemarin, Gernas Rana hingga kebakaran Gunung Soputan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:35:14 +0700</t>
+          <t>Wed, 05 Aug 2026 06:33:15 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo, menetapkan Kepala Bagian (Kabag) Keuangan sekretariat DPRD setempat ...</t>
+          <t>Sejumlah berita humaniora kemarin yang masih menarik untuk dibaca, mulai dari Gernas Rana enam kementerian hingga ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5679951/kabag-keuangan-dprd-ponorogo-tersangka-korupsi-tunjangan-perumahan</t>
+          <t>https://www.antaranews.com/berita/5680192/humaniora-kemarin-gernas-rana-hingga-kebakaran-gunung-soputan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_23_53_24.Still477.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000141203_1.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -672,28 +672,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kemarin, Febrie ajukan praperadilan hingga nasib status jaksanya</t>
+          <t>Spotify sudah punya 300 juta pelanggan Premium</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:28:47 +0700</t>
+          <t>Wed, 05 Aug 2026 06:32:57 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Berbagai kabar hukum telah diwartakan Kantor Berita ANTARA pada Selasa (4/8), mulai dari mantan Jampidsus Febrie ...</t>
+          <t>Spotify dalam laporan keuangan terbarunya menyatakan bahwa layanan streaming-nya kini sudah memiliki 300 juta pelanggan ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680172/kemarin-febrie-ajukan-praperadilan-hingga-nasib-status-jaksanya</t>
+          <t>https://www.antaranews.com/berita/5680189/spotify-sudah-punya-300-juta-pelanggan-premium</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087202.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/01/27/logo-spotify.jpeg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -705,33 +705,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jetour bakal hadirkan lebih banyak pilihan NEV ke pasar Indonesia</t>
+          <t>BMKG: Sebagian besar Jakarta cerah pada Rabu pagi</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:24:54 +0700</t>
+          <t>Wed, 05 Aug 2026 06:09:43 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Jenama mobil listrik asal China, Jetour bakal hadirkan lebih banyak pilihan kendaraan energi baru (NEV) ke pasar . ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan sebagian besar wilayah DKI Jakarta cerah pada Rabu ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5680169/jetour-bakal-hadirkan-lebih-banyak-pilihan-nev-ke-pasar-indonesia</t>
+          <t>https://www.antaranews.com/berita/5680187/bmkg-sebagian-besar-jakarta-cerah-pada-rabu-pagi</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/WhatsApp-Image-2026-05-27-at-17.54.18.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/08/29/20221125_Monasberawan.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -748,28 +748,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OJK bantah alami defisit anggaran dalam laporan keuangan 2025</t>
+          <t>Kinerja KPK semester I-2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:16:57 +0700</t>
+          <t>Wed, 05 Aug 2026 06:00:00 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wakil Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Hernawan Bekti Sasongko membantah adanya isu defisit ...</t>
+          <t>Komisi Pemberantasan Korupsi (Dewas KPK) melakukan ribuan penindakan kasus tindak pidana korupsi selama semester ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680167/ojk-bantah-alami-defisit-anggaran-dalam-laporan-keuangan-2025</t>
+          <t>https://www.antaranews.com/infografik/5679727/kinerja-kpk-semester-i-2026</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/31b157c6-a45a-436b-8256-05aff0c845e7.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/20260804-Kinerja-KPK-semester-I-2026.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -786,28 +786,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gempa M 5,6 guncang barat laut Halmahera Barat, tak berpotensi tsunami</t>
+          <t>Kemendagri godok usulan DAU bayar gaji PPPK di daerah</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 04:04:11 +0700</t>
+          <t>Wed, 05 Aug 2026 05:46:09 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) melaporkan gempa dengan magnitudo 5,6 mengguncang barat laut ...</t>
+          <t>Kementerian Dalam Negeri (Kemendagri) masih menggodok usulan penggunaan Dana Alokasi Umum (DAU) untuk membantu ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680163/gempa-m-56-guncang-barat-laut-halmahera-barat-tak-berpotensi-tsunami</t>
+          <t>https://www.antaranews.com/berita/5680183/kemendagri-godok-usulan-dau-bayar-gaji-pppk-di-daerah</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/ilustrasi-gempa-3.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/raker-komisi-ii-dpr-dengan-kemendagri.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -824,28 +824,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Potret gelombang panas dan karhutla di Eropa</t>
+          <t>Vedanta Aluminium Laporkan Rekor Kinerja Q1 FY27; Laba Melonjak 205%, EBITDA Lebih dari Dua Kali Lipat Laporkan Rekor Kinerja Q1 FY27; Laba Melonjak 205%, EBITDA Lebih dari Dua Kali Lipat</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 03:29:29 +0700</t>
+          <t>Wed, 05 Aug 2026 05:43:00 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Eropa sedang menghadapi gelombang panas berkepanjangan dan kekeringan yang meluas. Kondisi tersebut semakin menambah ...</t>
+          <t>- Vedanta Aluminium Metal Limited (NSE: VAML, BSE: 544780), salah satu produsen aluminium terkemuka di dunia, hari ini ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680159/potret-gelombang-panas-dan-karhutla-di-eropa</t>
+          <t>https://www.antaranews.com/berita/5680180/vedanta-aluminium-laporkan-rekor-kinerja-q1-fy27-laba-melonjak-205-ebitda-lebih-dari-dua-kali-lipat-laporkan-rekor-kinerja-q1-fy27-laba-melonjak-205-ebitda-lebih-dari-dua-kali-lipat</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000022_20260804_CBMFN0A001.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/03/23/Logo-BusinessWire-800x600.jpg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -862,28 +862,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bluebird bukukan pendapatan Rp2,97 triliun di Semester I 2026</t>
+          <t>Lucho ungkap suka cita Persib Bandung lolos ke final Piala Presiden</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 03:02:51 +0700</t>
+          <t>Wed, 05 Aug 2026 05:25:35 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PT Blue Bird Tbk (Bird) membukukan pendapatan sebesar Rp2,97 triliun pada Semester I 2026, didukung kinerja seluruh ...</t>
+          <t>Gelandang Persib Bandung Luciano Guaycochea atau yang kerap disapa Lucho mengungkapkan suka cita timnya berhasil lolos ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680157/bluebird-bukukan-pendapatan-rp297-triliun-di-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5680179/lucho-ungkap-suka-cita-persib-bandung-lolos-ke-final-piala-presiden</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/B0EE512C-6D50-4F78-AADA-5319D04B8721.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/24/Persib-Bandung-Imbang-Lawan-Arema-FC-240426-DAN-04.jpg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -900,28 +900,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
+          <t>Kemarin, surpres penggantian Kapolri hingga harga BBM subsidi tak naik</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
+          <t>Wed, 05 Aug 2026 04:58:19 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
+          <t>Berbagai kabar politik telah diwartakan Kantor Berita ANTARA pada Selasa (4/8), mulai dari Komisi III membantah adanya ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
+          <t>https://www.antaranews.com/berita/5680176/kemarin-surpres-penggantian-kapolri-hingga-harga-bbm-subsidi-tak-naik</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1001272341_1.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -938,28 +938,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
+          <t>Kabag Keuangan DPRD Ponorogo tersangka korupsi tunjangan perumahan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
+          <t>Wed, 05 Aug 2026 04:35:14 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
+          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo, menetapkan Kepala Bagian (Kabag) Keuangan sekretariat DPRD setempat ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
+          <t>https://www.antaranews.com/video/5679951/kabag-keuangan-dprd-ponorogo-tersangka-korupsi-tunjangan-perumahan</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_23_53_24.Still477.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -976,28 +976,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
+          <t>Kemarin, Febrie ajukan praperadilan hingga nasib status jaksanya</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
+          <t>Wed, 05 Aug 2026 04:28:47 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
+          <t>Berbagai kabar hukum telah diwartakan Kantor Berita ANTARA pada Selasa (4/8), mulai dari mantan Jampidsus Febrie ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
+          <t>https://www.antaranews.com/berita/5680172/kemarin-febrie-ajukan-praperadilan-hingga-nasib-status-jaksanya</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087202.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1009,33 +1009,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
+          <t>Jetour bakal hadirkan lebih banyak pilihan NEV ke pasar Indonesia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
+          <t>Wed, 05 Aug 2026 04:24:54 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
+          <t>Jenama mobil listrik asal China, Jetour bakal hadirkan lebih banyak pilihan kendaraan energi baru (NEV) ke pasar . ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
+          <t>https://otomotif.antaranews.com/berita/5680169/jetour-bakal-hadirkan-lebih-banyak-pilihan-nev-ke-pasar-indonesia</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/WhatsApp-Image-2026-05-27-at-17.54.18.jpeg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1052,28 +1052,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
+          <t>OJK bantah alami defisit anggaran dalam laporan keuangan 2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
+          <t>Wed, 05 Aug 2026 04:16:57 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
+          <t>Wakil Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Hernawan Bekti Sasongko membantah adanya isu defisit ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
+          <t>https://www.antaranews.com/berita/5680167/ojk-bantah-alami-defisit-anggaran-dalam-laporan-keuangan-2025</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/31b157c6-a45a-436b-8256-05aff0c845e7.jpeg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1090,28 +1090,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
+          <t>Gempa M 5,6 guncang barat laut Halmahera Barat, tak berpotensi tsunami</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
+          <t>Wed, 05 Aug 2026 04:04:11 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) melaporkan gempa dengan magnitudo 5,6 mengguncang barat laut ...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
+          <t>https://www.antaranews.com/berita/5680163/gempa-m-56-guncang-barat-laut-halmahera-barat-tak-berpotensi-tsunami</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/ilustrasi-gempa-3.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1128,28 +1128,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
+          <t>Potret gelombang panas dan karhutla di Eropa</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
+          <t>Wed, 05 Aug 2026 03:29:29 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
+          <t>Eropa sedang menghadapi gelombang panas berkepanjangan dan kekeringan yang meluas. Kondisi tersebut semakin menambah ...</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
+          <t>https://www.antaranews.com/berita/5680159/potret-gelombang-panas-dan-karhutla-di-eropa</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/CjkinzN000022_20260804_CBMFN0A001.jpg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1166,28 +1166,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
+          <t>Bluebird bukukan pendapatan Rp2,97 triliun di Semester I 2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
+          <t>Wed, 05 Aug 2026 03:02:51 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
+          <t>PT Blue Bird Tbk (Bird) membukukan pendapatan sebesar Rp2,97 triliun pada Semester I 2026, didukung kinerja seluruh ...</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
+          <t>https://www.antaranews.com/berita/5680157/bluebird-bukukan-pendapatan-rp297-triliun-di-semester-i-2026</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/B0EE512C-6D50-4F78-AADA-5319D04B8721.jpeg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1204,28 +1204,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
+          <t>Manajemen Orderkuota ajak masyarakat tak tertipu kontak palsu</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
+          <t>Wed, 05 Aug 2026 02:08:04 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
+          <t>Manajemen aplikasi Orderkuota mengajak masyarakat agar tidak tertipu dengan kontak palsu Contact Service (CS) yang ...</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
+          <t>https://www.antaranews.com/berita/5680156/manajemen-orderkuota-ajak-masyarakat-tak-tertipu-kontak-palsu</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/43bbb5ec-35e4-42b9-a62b-818e0a7433cc.jpeg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1242,28 +1242,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
+          <t>Wed, 05 Aug 2026 01:48:33 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang ...</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
+          <t>https://www.antaranews.com/video/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1280,28 +1280,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
+          <t>KPK pantau usulan pembentukan badan khusus pengelola aset rampasan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
+          <t>Wed, 05 Aug 2026 01:28:49 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) mengaku tengah memantau usulan pembentukan badan khusus yang bertindak sebagai ...</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
+          <t>https://www.antaranews.com/berita/5680153/kpk-pantau-usulan-pembentukan-badan-khusus-pengelola-aset-rampasan</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_7412.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1318,28 +1318,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>KPK sebut ada tiga sprindik pengembangan kasus KPP Banjarmasin</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
+          <t>Wed, 05 Aug 2026 01:19:17 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) menyebut ada tiga surat perintah penyidikan (sprindik) terkait pengembangan kasus ...</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680149/kpk-sebut-ada-tiga-sprindik-pengembangan-kasus-kpp-banjarmasin</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/pemeriksaan-lanjutan-mantan-kepala-kpp-madya-banjarmasin-2788325.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1356,28 +1356,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
+          <t>Indonesia kecam serangan Israel yang hambat rencana perdamaian Gaza</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
+          <t>Wed, 05 Aug 2026 01:16:54 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
+          <t>Indonesia mengecam keras serangan militer Israel ke Gaza, termasuk serangan terhadap rakyat sipil dan infrastruktur ...</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
+          <t>https://www.antaranews.com/berita/5680148/indonesia-kecam-serangan-israel-yang-hambat-rencana-perdamaian-gaza</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_6642b80a1e35b43f1ed5cb324e0b724b.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1394,28 +1394,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
+          <t>OJK terima 343 konsultasi calon peserta regulatory sandbox</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
+          <t>Wed, 05 Aug 2026 01:11:57 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan telah menerima sebanyak 343 kali permintaan konsultasi dari calon peserta ...</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
+          <t>https://www.antaranews.com/berita/5680144/ojk-terima-343-konsultasi-calon-peserta-regulatory-sandbox</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/d0f9bd15-895f-4b4c-92cb-60710e629f27.jpeg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1432,28 +1432,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
+          <t>KAI pastikan data digital pelanggan tetap aman dan terlindungi</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
+          <t>Wed, 05 Aug 2026 00:59:43 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
+          <t>PT Kereta Api Indonesia (Persero) memastikan data digital pelanggan tetap aman dan terlindungi, serta terjaga ...</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
+          <t>https://www.antaranews.com/berita/5680143/kai-pastikan-data-digital-pelanggan-tetap-aman-dan-terlindungi</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/B0F7D95A-7D7F-48C9-8968-B0DDC05BDC2B.jpeg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1465,33 +1465,33 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
+          <t>Ajax resmi umumkan kedatangan Marc ter Stegen</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:36:51 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>Klub Liga Belanda Ajax resmi mengumumkan kedatangan penjaga gawang senior Marc-Andre ter Stegen dari klub Liga Spanyol ...</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
+          <t>https://www.antaranews.com/berita/5680139/ajax-resmi-umumkan-kedatangan-marc-ter-stegen</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/image-36.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1503,33 +1503,33 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:28:16 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku ...</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/video/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1541,33 +1541,33 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
+          <t>Pol Espargaro gantikan Maverick Vinales di KTM untuk MotoGP Inggris</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:27:29 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>Pembalap cadangan Pol Espargaro akan menggantikan Maverick Vinales membela tim Red Bull KTM Tech3 untuk bertarung pada ...</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
+          <t>https://www.antaranews.com/berita/5680135/pol-espargaro-gantikan-maverick-vinales-di-ktm-untuk-motogp-inggris</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/07/11/804ab04d-3317-45c3-9b93-28f5a08b0d9a.jpeg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1579,33 +1579,33 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
+          <t>OJK Cirebon bantu petambak garam akses pembiayaan sesuai musim panen</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:23:49 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
+          <t>Kantor Otoritas Jasa Keuangan (OJK) Cirebon membantu petambak garam Kabupaten Cirebon, Jawa Barat, memperoleh akses ...</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
+          <t>https://www.antaranews.com/berita/5680133/ojk-cirebon-bantu-petambak-garam-akses-pembiayaan-sesuai-musim-panen</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001518164.jpg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1617,33 +1617,33 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:22:20 +0700</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran ...</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
+          <t>https://www.antaranews.com/video/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1655,33 +1655,33 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
+          <t>47 pemain bela Indonesia di Srikandi Merdeka Cup 2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:15:05 +0700</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
+          <t>Sebanyak 47 pemain diumumkan akan membela timnas kelompok umur U18 putri Indonesia yang akan bertarung di kompetisi ...</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
+          <t>https://www.antaranews.com/berita/5680132/47-pemain-bela-indonesia-di-srikandi-merdeka-cup-2026</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/02/Latihan-Timnas-Putri-U17-020526-Ada-1A.jpg</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1693,33 +1693,33 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
+          <t>Raisa akan nyanyikan "Cahaya Hati" dalam Hikayat Srikandi Nusantara</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:09:20 +0700</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
+          <t>Penyanyi Raisa akan membawakan lagu "Cahaya Hati" untuk pertama kalinya di hadapan publik dalam Pagelaran ...</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
+          <t>https://www.antaranews.com/berita/5680127/raisa-akan-nyanyikan-cahaya-hati-dalam-hikayat-srikandi-nusantara</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975376_w.jpg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1731,33 +1731,33 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
+          <t>Yura sebut Pagelaran Sabang Merauke jadi ruang untuk eksplorasi diri</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 00:01:57 +0700</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
+          <t>Penyanyi Yura Yunita mengatakan Pagelaran Sabang Merauke bertajuk "Hikayat Srikandi Nusantara" menjadi ruang ...</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
+          <t>https://www.antaranews.com/berita/5680119/yura-sebut-pagelaran-sabang-merauke-jadi-ruang-untuk-eksplorasi-diri</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/photo_6309921447844975416_w.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1774,28 +1774,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
+          <t>Latihan trimatra TNI, 27 personel KDOL terjun di Dabo Singkep Kepri</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
+          <t>ANTARA - TNI menggelar latihan terintegrasi trimatra melalui penerjunan Kelompok Depan Operasi Lintas Udara (KDOL) yang melibatkan 27 personel, di sekitar Drop Zone Bandara Dabo Singkep, Kepulauan Riau Selasa (4/8). Kapuspen TNI Mayjen Muhammad Nas menyebutkan, rangkaian kegiatan ini akan dilakukan selama dua hari dengan melibatkan lebih dari 12 ribu personel, sebagai wujud profesionalisme pelaksanaan tugas menjaga kedaulatan NKRI hingga pulau terpencil. (Angiela Chantiequ/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
+          <t>https://www.antaranews.com/berita/5680155/latihan-trimatra-tni-27-personel-kdol-terjun-di-dabo-singkep-kepri</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/LATIHAN-TRIMATRA-TNI-27-PERSONEL-KDOL-TERJUN-DI-DABO-SINGKEP-KEPRI.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1812,28 +1812,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
+          <t>KNKT mulai investigasi kebakaran KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
+          <t>ANTARA - Wakil Menteri Perhubungan Suntana, Selasa (4/8), menyatakan investigasi untuk mengetahui penyebab kebakaran Kapal Motor (KM) Mutiara Sentosa II telah dimulai. Ia memastikan akan ada sanksi bagi perusahaan pelayaran serta hukuman pidana jika dalam investigasi ditemukan unsur kelalaian dalam operasional kapal yang mengabaikan aspek keselamatan. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
+          <t>https://www.antaranews.com/berita/5680129/knkt-mulai-investigasi-kebakaran-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KNKT-MULI-INVESTIGASI-KEBAKARAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1850,28 +1850,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
+          <t>Inovasi pisang goreng kipas Pekanbaru tembus pasar ekspor</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Usaha Pisang Goreng Kipas Kuantan II di Kota Pekanbaru, Riau, mengembangkan produk setengah matang dan beku (frozen) sehingga berhasil menembus pasar ekspor. Pemilik usaha Yana Patriana mengatakan produknya kini rutin dipasarkan ke Australia, Malaysia, dan mulai diminati calon pembeli dari Jepang. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
+          <t>https://www.antaranews.com/berita/5680123/inovasi-pisang-goreng-kipas-pekanbaru-tembus-pasar-ekspor</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/INOVASI-PISANG-GORENG-KIPAS-PEKANBARU-TEMBUS-PASAR-EKSPOR.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1888,28 +1888,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
+          <t>KPK ungkap korupsi digitalisasi SPBU yang rugikan negara Rp322 M</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) telah menahan tiga orang yang ditetapkan sebagai tersangka dalam kasus dugaan korupsi digitalisasi Stasiun Pengisian Bahan Bakar Umum (SPBU) PT Pertamina (Persero). Plt. Direktur Penyidikan KPK Achmad Taufik Husein, di Jakarta, Selasa (4/8), menyebut kerugian negara akibat kasus ini mencapai Rp322,18 miliar. (Afra Augesti/Ryan Rahman/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
+          <t>https://www.antaranews.com/berita/5680104/kpk-ungkap-korupsi-digitalisasi-spbu-yang-rugikan-negara-rp322-m</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KPK-UNGKAP-KORUPSI-DIGITALISASI-SPBU-YANG-RUGIKAN-NEGARA-RP322-M.jpg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1926,28 +1926,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
+          <t>Pasca banjir 15 titik, Sumbar kerahkan alat berat pulihkan sungai</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Gubernur Sumatera Barat Mahyeldi Ansharullah mengatakan sejumlah alat berat telah dikerahkan dinas terkait untuk membantu penanganan sejumlah aliran sungai yang memicu banjir pada 15 titik dampak cuaca ekstrem di Kota Padang pada Senin (3/8). Saat meninjau lokasi bencana pada Selasa (4/8), Mahyeldi memastikan seluruh kebutuhan dasar masyarakat yang terdampak banjir terpenuhi dengan baik. (Fandi Yogari Saputra/Satrio Giri Marwanto/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
+          <t>https://www.antaranews.com/berita/5680097/pasca-banjir-15-titik-sumbar-kerahkan-alat-berat-pulihkan-sungai</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PASCA-BANJIR-15-TITIK-SUMBAR-KERAHKAN-ALAT-BERAT-PULIHKAN-SUNGAI.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1964,28 +1964,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
+          <t>BBKSDA Riau evaluasi penanganan gajah binaan usai kematian Jovi</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
+          <t>ANTARA - Balai Besar Konservasi Sumber Daya Alam (BBKSDA) Riau mengevaluasi pengelolaan dan pelayanan kesehatan gajah binaan setelah Gajah Jovi mati usai menjalani perawatan intensif selama 34 hari. Pelaksana Harian Kepala BBKSDA Riau Ujang Holisudin mengatakan hasil uji laboratorium akan menjadi dasar penyusunan langkah pencegahan dan peningkatan penanganan kesehatan gajah binaan. (Farah Khadija/Annisa Firdausi/Satrio Giri Marwanto/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
+          <t>https://www.antaranews.com/berita/5680077/bbksda-riau-evaluasi-penanganan-gajah-binaan-usai-kematian-jovi</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BBKSDA-RIAU-EVALUASI-PENANGANAN-GAJAH-BINAAN-USAI-KEMATIAN-JOVI.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2002,28 +2002,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
+          <t>Pemerintah tegaskan komitmen perlindungan anak melalui Gernas Rana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Pemerintah kembali menegaskan komitmen untuk memberikan perlindungan kepada anak, sekaligus membangun ruang digital yang aman bagi anak melalui Gerakan Nasional Ruang Aman dan Nyaman untuk Anak (GERNAS RANA). Menurut Menteri Koordinator bidang Pembangunan Manusia dan Kebudayaan Pratikno, di Jakarta, Selasa (4/8), GERNAS RANA diharapkan mampu melindungi anak di lingkungan keluarga, satuan pendidikan, ruang publik, dan ruang digital. (Afra Augesti/Ryan Rahman/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
+          <t>https://www.antaranews.com/berita/5680069/pemerintah-tegaskan-komitmen-perlindungan-anak-melalui-gernas-rana</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/PEMERINTAH-TEGASKAN-KOMITMEN-PERLINDUNGAN-ANAK-MELALUI-GERNAS-RANA.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2040,28 +2040,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kabag Keuangan DPRD Ponorogo tersangka korupsi tunjangan perumahan</t>
+          <t>Polda Babel tahan tiga tersangka kasus korupsi alat kedokteran</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo, menetapkan Kepala Bagian (Kabag) Keuangan sekretariat DPRD setempat sebagai tersangka dalam kasus dugaan korupsi tunjangan perumahan anggota DPRD setempat, yang merugikan negara hingga 3,6 miliar rupiah. (Rindhu Dwi Kartiko/Arif Prada/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Direktorat Reserse Kriminal Khusus (Ditreskrimsus) Polda Kepulauan Bangka Belitung menahan tiga tersangka dalam perkara dugaan korupsi pengadaan belanja modal alat kedokteran umum atau Medical Operational Tools (MOT) di RSUD Dr. (HC) Ir. Soekarno Tahun Anggaran 2021. Ketiga tersangka masing-masing berinisial AH selaku Pejabat Pembuat Komitmen (PPK), AY selaku Direktur PT BWH sebagai penyedia, serta H selaku Direktur PT RDP yang berperan sebagai perusahaan pendukung. (Chandrika Purnama Dewi/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679951/kabag-keuangan-dprd-ponorogo-tersangka-korupsi-tunjangan-perumahan</t>
+          <t>https://www.antaranews.com/berita/5680057/polda-babel-tahan-tiga-tersangka-kasus-korupsi-alat-kedokteran</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_23_53_24.Still477.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLDA-BABEL-TAHAN-TIGA-TERSANGKA-KASUS-KORUPSI-ALAT-KEDOKTERAN.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2078,28 +2078,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
+          <t>Bahlil tegaskan pemegang IUPK batu bara wajib hilirisasi</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan perusahaan batu bara yang memperoleh Izin Usaha Pertambangan Khusus (IUPK) wajib menjalankan hilirisasi sesuai arahan Presiden Prabowo Subianto dan amanat Pasal 33 Undang-Undang Dasar 1945. (Cahya Sari/Irfansyah Naufal Nasution/Arif Prada/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
+          <t>https://www.antaranews.com/berita/5680043/bahlil-tegaskan-pemegang-iupk-batu-bara-wajib-hilirisasi</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_34_51_16.Still481.jpg</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2116,28 +2116,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
+          <t>Basarnas hentikan operasi kedaruratan KM Mutiara Sentosa II</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) menghentikan operasi kedaruratan Kapal Motor (KM) Mutiara Sentosa II, Selasa (4/8). Terdata total korban yang telah dievakuasi sebanyak 238 orang, lima di antaranya meninggal dunia. (Hanif Nasrullah/Soni Namura/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
+          <t>https://www.antaranews.com/berita/5680036/basarnas-hentikan-operasi-kedaruratan-km-mutiara-sentosa-ii</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/BASARNAS-HENTIKAN-OPERASI-KEDARURATAN-KM-MUTIARA-SENTOSA-II.jpg</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2154,28 +2154,28 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
+          <t>Kepala Bappisus tanggapi isu Surpres pergantian Kapolri</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
+          <t>ANTARA - Kepala Badan Pengendalian Pembangunan dan Investigasi Khusus (Bappisus) Aris Marsudiyanto, Selasa (4/8), merespons soal isu Surpres penggantian Kapolri. Menurutnya pergantian pucuk pimpinan Polri tergantung pada keputusan Presiden Prabowo Subianto. (Cahya Sari/Irfansyah Naufal Nasution/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
+          <t>https://www.antaranews.com/berita/5680031/kepala-bappisus-tanggapi-isu-surpres-pergantian-kapolri</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEPALA-BAPPISUS-TANGGAPI-ISU-SURPRES-PERGANTIAN-KAPOLRI.jpg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2192,28 +2192,28 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
+          <t>Palestina gelar pemakaman massal 112 jenazah korban serangan Israel</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+          <t>ANTARA - Ribuan warga Palestina di Gaza pada Selasa (4/8) melaksanakan shalat jenazah sekaligus pemakaman massal untuk 112 korban yang tewas akibat perang Israel. Para korban tersebut sebelumnya dievakuasi dari bawah reruntuhan bangunan yang hancur. (ANADOLU/ Winanto/Arif Prada/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+          <t>https://www.antaranews.com/berita/5680009/palestina-gelar-pemakaman-massal-112-jenazah-korban-serangan-israel</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_32_00_18.Still480.jpg</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2230,28 +2230,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+          <t>Kemnaker: Pendaftar magang nasional tembus 400 ribu orang</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+          <t>ANTARA - Menteri Ketenagakerjaan Yassierli mengatakan jumlah pendaftar program magang nasional tembus lebih dari 400 ribu orang dari kuota awal sebanyak 50 ribu peserta. Menaker di Makassar, Sulawesi Selatan, Selasa (4/8) menyebut pihaknya juga terus memperluas pelatihan vokasi, sebagai upaya meningkatkan kualitas sumber daya manusia. (Shintia Aryanti Krisna/Chairul Fajri/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+          <t>https://www.antaranews.com/berita/5679976/kemnaker-pendaftar-magang-nasional-tembus-400-ribu-orang</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEMNAKER-PENDAFTAR-MAGANG-NASIONAL-TEMBUS-400-RIBU-ORANG.jpg</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2268,28 +2268,28 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+          <t>Pemkot Semarang seleksi UMKM dan IKM untuk pembinaan lanjutan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+          <t>ANTARA - Wali Kota Semarang Agustina Wilujeng Pramestuti menyebut bahwa saat ini pemerintah tengah melakukan sensus dan seleksi terhadap para Pelaku Usaha Mikro, Kecil, dan Menengah (UMKM) dan Industri Kecil dan Menengah (IKM) untuk dilakukan pembinaan lebih lanjut. Dari 3.000 lebih UMKM di Kota Semarang, hingga saat ini telah ada 200 lebih yang terseleksi, dan 11 di antaranya telah memenuhi syarat untuk dilakukan pembinaan lanjutan. (Fx. Suryo Wicaksono/Arif Prada/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+          <t>https://www.antaranews.com/berita/5679967/pemkot-semarang-seleksi-umkm-dan-ikm-untuk-pembinaan-lanjutan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_26_34_14.Still478.jpg</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2306,28 +2306,28 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+          <t>Polres Cilegon siagakan posko terpadu hadapi ancaman musim kemarau</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Polres Cilegon membentuk posko terpadu bersama Pemerintah Kota Cilegon, TNI, Badan Penanggulangan Bencana Daerah (BPBD), Dinas Pemadam Kebakaran, dan instansi terkait untuk memperkuat kesiapsiagaan menghadapi potensi kebakaran dan krisis air bersih selama musim kemarau. Kapolres Cilegon AKBP Moehamad Probandono Bobby Danuardi mengatakan pada Selasa (4/8), posko tersebut disiapkan untuk mempercepat penanganan keadaan darurat di wilayah Kota Cilegon. (Susmiatun Hayati/Soni Namura/Arsy Fitriady)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+          <t>https://www.antaranews.com/berita/5679961/polres-cilegon-siagakan-posko-terpadu-hadapi-ancaman-musim-kemarau</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/POLRES-CILEGON-SIAGAKAN-POSKO-TERPADU-HADAPI-ANCAMAN-MUSIM-KEMARAU.jpg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2344,28 +2344,28 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+          <t>Kabag Keuangan DPRD Ponorogo tersangka korupsi tunjangan perumahan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo, menetapkan Kepala Bagian (Kabag) Keuangan sekretariat DPRD setempat sebagai tersangka dalam kasus dugaan korupsi tunjangan perumahan anggota DPRD setempat, yang merugikan negara hingga 3,6 miliar rupiah. (Rindhu Dwi Kartiko/Arif Prada/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+          <t>https://www.antaranews.com/berita/5679951/kabag-keuangan-dprd-ponorogo-tersangka-korupsi-tunjangan-perumahan</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_23_53_24.Still477.jpg</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2382,28 +2382,28 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+          <t>Pemkot Solo tegaskan tak ada toleransi bagi penjual miras tanpa izin</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+          <t>ANTARA - Wali Kota Solo Respati Ardi menegaskan tidak ada toleransi bagi peredaran minuman keras (miras) tanpa izin. Respati menyebut pihaknya mengambil langkah cepat berupa penertiban ketat, penyitaan ratusan botol, hingga penutupan tempat usaha yang melanggar aturan. Hal tersebut disampaikan Respati saat ditemui di Balai Kota Solo pada Selasa (4/8). (Denik Apriyani/Arif Prada/Roy Rosa Bachtiar)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+          <t>https://www.antaranews.com/berita/5679915/pemkot-solo-tegaskan-tak-ada-toleransi-bagi-penjual-miras-tanpa-izin</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_19_16_29.Still476.jpg</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2420,28 +2420,28 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+          <t>Kekeringan makin meluas, BPBD Jember distribusi air hingga perbukitan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Badan Penanggulangan Bencana Daerah Kabupaten Jember mendistribusikan air bersih berikut tandon dari kawasan kota hingga perbukitan di wilayah Desa Mulyorejo, Kecamatan Silo pada Selasa (4/8). Langkah tersebut dilakukan dalam rangka mengatasi kekeringan yang semakin meluas dari yang sebelumnya berdampak kepada 125 kepala keluarga (KK) kini menjadi 535 KK.  (Hamka Agung Balya/Chairul Fajri/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+          <t>https://www.antaranews.com/berita/5679911/kekeringan-makin-meluas-bpbd-jember-distribusi-air-hingga-perbukitan</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/KEKERINGAN-MAKIN-MELUAS-BPBD-JEMBER-DISTRIBUSI-AIR-HINGGA-PERBUKITAN.jpg</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2458,28 +2458,28 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+          <t>Patung marmer monumental berusia 2.500 tahun ditemukan di Turki</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Patung marmer monumental berusia 2.500 tahun telah ditemukan di kota kuno Sardes di Turki barat. Penemuan tersebut diumumkan oleh Menteri Kebudayaan dan Pariwisata Turki Mehmet Nuri Ersoy pada Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Arif Prada/Winanto)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+          <t>https://www.antaranews.com/berita/5679880/patung-marmer-monumental-berusia-2500-tahun-ditemukan-di-turki</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Sequence-13.13_17_23_01.Still475.jpg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2496,333 +2496,333 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+          <t>Pemerintah tangani persoalan listrik di Kalimantan secara terukur</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
+          <t>ANTARA - Menteri ESDM Bahlil Lahadalia, Selasa (4/8), memastikan penanganan permasalahan listrik di wilayah Kalimantan dilakukan secara cepat dan terukur. Menurutnya, pemadaman listrik di wilayah tersebut terjadi karena pemeliharaan jaringan induk, bukan persoalan pasokan energi. (Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679867/pemerintah-tangani-persoalan-listrik-di-kalimantan-secara-terukur</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TANGANI-PERSOALAN-LISTRIK-DI-KALIMANTAN-SECARA-TERUKUR.jpg</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Dinkes Lhokseumawe uji kualitas air cegah pencemaran E. coli</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Kesehatan Kota Lhokseumawe, Aceh, menguji kualitas air baku di Desa Pusong Baru, Kecamatan Banda Sakti, sebagai langkah mencegah risiko pencemaran bakteri Escherichia coli (E. coli). Pemeriksaan dilakukan menyusul kekhawatiran warga terhadap kondisi lingkungan yang dipenuhi sampah dan saluran pembuangan yang tersumbat. (Try Vanny S/Soni Namura/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679864/dinkes-lhokseumawe-uji-kualitas-air-cegah-pencemaran-e-coli</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/DINKES-LHOKSEUMAWE-UJI-KUALITAS-AIR-CEGAH-PENCEMARAN-E.COLI.jpg</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Pemkot Solo siapkan museum Brigjen Slamet Riyadi untuk edukasi sejarah</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Solo merehabilitasi rumah masa kecil Pahlawan Nasional Brigjen Slamet Riyadi di Kampung Joyosuran, Kecamatan Pasar Kliwon. Bangunan bersejarah tersebut akan difungsikan sebagai museum dan rumah singgah guna memperluas edukasi sejarah bagi masyarakat, khususnya pelajar. (Denik Apriyani/Andi Bagasela/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679839/pemkot-solo-siapkan-museum-brigjen-slamet-riyadi-untuk-edukasi-sejarah</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKOT-SOLO-SIAPKAN-MUSEUM-BRIGJEN-SLAMET-RIYADI-UNTUK-EDUKASI-SEJARAH.jpg</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Kemenkes berkomitmen jaga harapan hidup lewat cek kesehatan gratis</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Kesehatan mencatat sebanyak 73 juta masyarakat telah mengikuti program Cek Kesehatan Gratis hingga 31 Juli 2026. Saat ditemui di Jakarta Selasa (4/7), Direktur Jenderal Kesehatan Primer dan Komunitas Kemenkes Maria Endang Sumiwi menjelaskan program tersebut diharapkan memperkuat deteksi dini penyakit sekaligus mendukung peningkatan angka harapan hidup masyarakat Indonesia yang kini mencapai 74 tahun. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679821/kemenkes-berkomitmen-jaga-harapan-hidup-lewat-cek-kesehatan-gratis</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-201356.jpg</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Jelang HUT RI, pedagang bendera di Palangka Raya panen rezeki</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ANTARA - Menjelang peringatan Hari Ulang Tahun (HUT) ke-81 Kemerdekaan Republik Indonesia, pedagang bendera Merah Putih dan pernak-pernik bernuansa kemerdekaan mulai bermunculan di sejumlah ruas jalan protokol di Kota Palangka Raya, Kalimantan Tengah, Selasa (4/8). Salah satu pedagang musiman tersebut diketahui berasal dari Bandung, Jawa Barat, yang datang setiap tahun untuk memanen rezeki.(Redianto Tumon Sp/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679807/jelang-hut-ri-pedagang-bendera-di-palangka-raya-panen-rezeki</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_JELANG-HUT-RI-PEDAGANG-BENDERA-DI-PALANGKA-RAYA-PANEN-REZEKI.jpg</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BPJS Kesehatan luncurkan NADI JKN untuk aktifkan 54 juta peserta</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ANTARA - Badan Penyelenggara Jaminan Sosial (BPJS) Kesehatan meluncurkan program Menabung Demi Iuran Jaminan Kesehatan Nasional (NADI JKN) sebagai upaya mengaktifkan kembali sekitar 54 juta peserta yang menunggak iuran. Program yang dirilis Selasa (4/7) diharapkan memperluas kepesertaan aktif sekaligus menjaga keberlanjutan pembiayaan JKN. (Nico Anggriawan/Rizky Bagus Dhermawan/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679785/bpjs-kesehatan-luncurkan-nadi-jkn-untuk-aktifkan-54-juta-peserta</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-194723.jpg</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>CdM Indonesia targetkan tim bulu tangkis boyong emas di Asian Games</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ANTARA - Chef de Mission (Cdm) Indonesia, Todutua Pasaribu menyambangi tempat pelatihan nasional cabang olahraga bulu tangkis Pelatnas (PBSI) di Jakarta, Selasa (4/26). Todutua menargetkan cabang olahraga bulu tangkis dapat meraih medali emas pada ajang Asian Games 2026. (Ibnu Zaki/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679745/cdm-indonesia-targetkan-tim-bulu-tangkis-boyong-emas-di-asian-games</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_CDM-INDONESIA-TARGETKAN-TIM-BULU-TANGKIS-BOYONG-EMAS-DI-ASIAN-GAMES.jpg</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>DLH Cilegon tagih piutang retribusi sampah Kab. Serang sebesar Rp1,3 M</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Lingkungan Hidup (DLH) Kota Cilegon, Selasa (4/8), melayangkan tagihan pembayaran persampahan kepada Dinas Lingkungan Hidup Kabupaten Serang yang memiliki piutang pembayaran retribusi sampah sebesar Rp1,3 miliar. Dinas Lingkungan Hidup Kota Cilegon, menyebutkan, piutang itu berasal akibat pembayaran kewajiban retribusi sampah yang tidak dibayarkan pada Desember 2023 dan Januari 2024 lalu. (Susmiatun Hayati/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679737/dlh-cilegon-tagih-piutang-retribusi-sampah-kab-serang-sebesar-rp13-m</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DLH-CILEGON-TAGIH-PIUTANG-RETRIBUSI-SAMPAH-KAB.SERANG-SEBESAR-RP1-3-M.jpg</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo antar langsung kepulangan PM Thailand dari Halim</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
           <t>ANTARA - Presiden RI Prabowo Subianto mengantar langsung kepulangan Perdana Menteri Thailand Anutin Charnvirakul dari Lanud Halim Perdanakusuma, Jakarta, Selasa (4/8). Kepulangan PM Anutin menutup rangkaian kunjungannya di Indonesia selama dua hari yang memperkuat kemitraan strategis kedua negara di sektor keamanan, ekonomi, hingga energi.
 (Cahya Sari/Irfansyah Naufal Nasution/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679719/presiden-prabowo-antar-langsung-kepulangan-pm-thailand-dari-halim</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-192451.jpg</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2839,28 +2839,28 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
+          <t>Pemerintah dorong percepatan proyek PSEL di Makassar</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah pusat kembali menegaskan komitmennya dalam mempercepat pembangunan Pengolahan Sampah menjadi Energi Listrik (PSEL) di Kota Makassar sebagai bagian dari upaya penanganan darurat sampah nasional. Menteri Koordinator Bidang Pangan, Zulkifli Hasan, menyatakan bahwa pemerintah memberi tenggat waktu dua pekan untuk penyelesaian berbagai kendala proyek tersebut. Jika tidak ada kemajuan, Pemerintah Provinsi Sulawesi Selatan diminta mengambil alih proses percepatannya. (Shintia Aryanti Krisna/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
+          <t>https://www.antaranews.com/berita/5679705/pemerintah-dorong-percepatan-proyek-psel-di-makassar</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-184835_1.jpg</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2877,28 +2877,28 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
+          <t>Pemprov Kalsel gandeng 46 perusahaan, hadirkan 1.145 lowongan kerja</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+          <t>ANTARA - Pemerintah Provinsi Kalimantan Selatan menyelenggarakan bursa kerja 2026 selama empat hari dari tanggal 3-6 Agustus 2026 di Gedung Sultan Adam Kayu Tangi Banjarmasin. Pada agenda tersebut, Pemprov Kalsel menggandeng 46 perusahaan untuk menyediakan 1,145 lowongan pekerjaan.(Latif Thohir/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
+          <t>https://www.antaranews.com/berita/5679669/pemprov-kalsel-gandeng-46-perusahaan-hadirkan-1145-lowongan-kerja</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMPROV-KALSEL-GANDENG-46-PERUSAHAAN-HADIRKAN-1.145-LOWONGAN-KERJA.jpg</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2915,28 +2915,28 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
+          <t>Prabowo instruksikan harga BBM nonsubsidi diturunkan ikuti harga dunia</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Presiden Prabowo Subianto menginstruksikan agar harga BBM nonsubsidi dapat disesuaikan seiring menurunnya harga minyak dunia. Hal itu disampaikan Menteri ESDM Bahlil Lahadalia, Selasa (4/8), usai menghadiri ratas bersama Presiden di Istana Kepresidenan, Jakarta.(Cahya Sari/Irfansyah Naufal Nasution/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
+          <t>https://www.antaranews.com/berita/5679649/prabowo-instruksikan-harga-bbm-nonsubsidi-diturunkan-ikuti-harga-dunia</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PRABOWO-INSTRUKSIKAN-HARGA-BBM-NONSUBSIDI-DITURUNKAN-IKUTI-HARGA-DUNIA.jpg</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2953,28 +2953,28 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
+          <t>BPBD Ngawi distribusikan air bersih ke 4 kecamatan atasi kekeringan</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
+          <t>ANTARA - Memasuki musim kemarau, Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Ngawi, telah mendistribusikan air bersih ke sejumlah desa yang ada di empat kecamatan. Distribusi air dilengkapi dengan tandon air atau terpal yang dibentuk menjadi kolam penampungan air sementara. (Rindhu Dwi Kartiko/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
+          <t>https://www.antaranews.com/berita/5679647/bpbd-ngawi-distribusikan-air-bersih-ke-4-kecamatan-atasi-kekeringan</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-183625.jpg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2991,28 +2991,28 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
+          <t>RI-Thailand perkuat kerja sama kemitraan strategis bidang pertahanan</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
+          <t>ANTARA - Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin dan Menteri Pertahanan Thailand Letnan Jenderal Adul Boonthumjaroen melangsungkan pertemuan di Jakarta, Selasa (4/8). Pada pertemuan tersebut Menhan Sjafrie menyampaikan kedua negara membahas kerja sama kemitraan strategis di bidang pertahanan.(Setyanka Harviana Putri/Irfan Hardiansah/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
+          <t>https://www.antaranews.com/berita/5679620/ri-thailand-perkuat-kerja-sama-kemitraan-strategis-bidang-pertahanan</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_RI-THAILAND-PERKUAT-KERJA-SAMA-KEMITRAAN-STRATEGIS-BIDANG-PERTAHANAN.jpg</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3029,343 +3029,647 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
+          <t>Alwi Farhan optimistis melaju jauh di Kejuaraan Dunia BWF New Delhi</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
+          <t>ANTARA - Pebulu tangkis tunggal putra Indonesia, Alwi Farhan, Selasa (4/7), menyatakan persiapan latihan menuju Kejuaraan Dunia BWF di New Delhi, India berjalan dengan baik. Meski tidak masuk dalam daftar unggulan, Alwi optimistis mampu memberikan perlawanan dan melaju jauh dalam turnamen akbar itu. (Rabitha El Adawiya/Ibnu Zaki/Rizky Bagus Dhermawan/Rijalul Vikry)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679613/alwi-farhan-optimistis-melaju-jauh-di-kejuaraan-dunia-bwf-new-delhi</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-181403_1.jpg</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>30 persen peserta pemagangan nasional di Kaltim direkrut perusahaan</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ANTARA - Program Pemagangan Nasional di Kalimantan Timur menjadi salah satu jalur penyerapan tenaga kerja. Dinas Tenaga Kerja dan Transmigrasi Kalimantan Timur mencatat sekitar 30 persen dari 1.000 peserta magang periode pertama tahun 2025 direkrut menjadi tenaga kerja di 150 perusahaan. (Hanifan Ma'ruf/Andi Bagasela/Arsy Fitriady)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679532/30-persen-peserta-pemagangan-nasional-di-kaltim-direkrut-perusahaan</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_30-PERSEN-PESERTA-PEMAGANGAN-NASIONAL-DI-KALTIM-DIREKRUT-PERUSAHAAN.jpg</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Menko Airlangga tegaskan ekonomi RI kuat hadapi gejolak global</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah memastikan kondisi ekonomi Indonesia masih berada pada jalur yang kuat, meski dihadapkan pada gejolak ekonomi global. Kepastian tersebut disampaikan Menteri Koordinator Bidang Perekonomian Airlangga Hartarto di Makassar, Sulsel, Selasa (4/8). Menurutnya fundamental ekonomi nasional masih terjaga yang tercermin dari laju inflasi yang menurun,hingga proyeksi pertumbuhan ekonomi yang tetap berada di atas 5 persen.(Shintia Aryanti Krisna/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679481/menko-airlangga-tegaskan-ekonomi-ri-kuat-hadapi-gejolak-global</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_MENKO-AIRLANGGA-TEGASKAN-EKONOMI-RI-KUAT-HADAPI-GEJOLAK-GLOBAL.jpg</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Polda Kalsel gagalkan peredaran 172,4 kg sabu jaringan lintas provinsi</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ANTARA - Ratusan kilogram sabu dan ratusan butir ekstasi berhasil disita oleh Kepolisian Daerah Kalimantan Selatan. Kapolda Kalsel Irjen Pol. Rosyanto Yudha Hermawan pada konferensi pers di Banjarbaru, Selasa (4/8) menyebut  sebagian barang bukti tersebut diduga terafiliasi dengan jaringan buronan kelas kakap Fredy Pratama.(Latif Thohir/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679459/polda-kalsel-gagalkan-peredaran-1724-kg-sabu-jaringan-lintas-provinsi</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-165304_1.jpg</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>DPRD Babel kawal dan cari solusi keluhan penambang rakyat</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ANTARA - Dewan Perwakilan Rakyat Daerah (DPRD) Provinsi Kepulauan Bangka Belitung menyatakan siap mengawal dan mencari solusi atas keluhan penambang rakyat setempat. Komitmen tersebut disampaikan Ketua DPRD Babel Didit Srigusjaya usai menggelar Rapat Dengar Pendapat (RDP) dengan Aliansi Tambang Rakyat di Pangkalpinang, pada Selasa (4/8). (Chandrika Purnama Dewi/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679449/dprd-babel-kawal-dan-cari-solusi-keluhan-penambang-rakyat</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_DPRD-BABEL-KAWAL-DAN-CARI-SOLUSI-KELUHAN-PENAMBANG-RAKYAT.jpg</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pemkab Banjarnegara salurkan Rp1,7 miliar bantuan pendidikan parpol</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, menyalurkan bantuan  keuangan sejumlah Rp1,7 miliar kepada 10 partai politik anggota parlemen. Anggaran tersebut bertujuan untuk pendidikan politik atau kaderisasi dan operasional internal organisasi sehingga bisa berdampak positif terhadap pembangunan daerah dengan adanya sinergi antara pemerintah dan parpol. (Addin Alfath Amajida/Andi Bagasela/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679435/pemkab-banjarnegara-salurkan-rp17-miliar-bantuan-pendidikan-parpol</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMKAB-BANJARNEGARA-SALURKAN-RP1-7-MILIAR-BANTUAN-PENDIDIKAN-PARPOL.jpg</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Jasa Marga jajaki kolaborasi edukasi transportasi di Museum Angkut</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ANTARA - ‎PT Jasa Marga (Persero) Tbk menjajaki kolaborasi dengan Museum Angkut Kota Batu, Selasa (4/8) untuk menghadirkan wahana edukasi transportasi yang modern dan interaktif. Kolaborasi ini akan menghadirkan pengalaman belajar mengenai keselamatan berkendara, rambu lalu lintas, hingga teknologi jalan tol. (Achmad Saif Hajarani/Rizky Bagus Dhermawan/Roy Rosa Bachtiar)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679417/jasa-marga-jajaki-kolaborasi-edukasi-transportasi-di-museum-angkut</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-164055.jpg</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Iran: Negosiasi dengan Oman fokus pada rute sementara di Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ANTARA - Negosiasi antara Iran dan Oman berfokus pada pencapaian kesepakatan tentang penetapan rute "sementara" untuk memastikan pelayaran yang aman di Selat Hormuz. Hal tersebut disampaikan Juru bicara Kementerian Luar Negeri Iran, Esmaeil Baghaei, pada  Senin (3/8). (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5679379/iran-negosiasi-dengan-oman-fokus-pada-rute-sementara-di-selat-hormuz</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-162550.jpg</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Pelantikan DHD 45, Gubernur Sumut tekankan semangat juang pahlawan</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
           <t>ANTARA - Dewan Harian Daerah (DHD) Badan Pembudayaan Kejuangan 45 Sumatera Utara resmi dilantik dan disaksikan langsung oleh Gubernur Sumatera Utara Bobby Nasution di Kantor Gubernur Sumut, Selasa, (4/8). Bobby menyebutkan tujuan dilantiknya DHD 45 Sumut ini untuk meneruskan semangat juang para pahlawan terdahulu agar tetap diterapkan hingga saat ini.
 (M. Valery Maulidzar S/Andi Bagasela/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679368/pelantikan-dhd-45-gubernur-sumut-tekankan-semangat-juang-pahlawan</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PELANTIKAN-DHD-45-GUBERNUR-SUMUT-TEKANKAN-SEMANGAT-JUANG-PAHLAWAN.jpg</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
         <is>
           <t>Kabut tebal hentikan lalu lintas maritim di Selat Bosporus Turki</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
         <is>
           <t>ANTARA - Lalu lintas maritim di Selat Bosporus Istanbul, Turki, dihentikan pada Senin (2/8) karena kabut tebal.Kabut tebal juga mengganggu layanan feri antara sisi Eropa dan Asia Istanbul, dengan feri penumpang dan kendaraan yang dihentikan hingga pemberitahuan lebih lanjut. (XINHUA/Ludmila Yusufin Diah Nastiti/Rizky Bagus Dhermawan/Winanto)</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679345/kabut-tebal-hentikan-lalu-lintas-maritim-di-selat-bosporus-turki</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-161506.jpg</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
         <is>
           <t>Mendag targetkan neraca dagang pada Juli 2026 kembali surplus</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Perdagangan Budi Santoso menargetkan neraca perdagangan Indonesia akan kembali mencetak surplus pada Juli 2026. Mendag di Jakarta pada Selasa (4/8) menyebut hal itu diproyeksikan seiring mulai stabilnya harga minyak dunia. (Sanya Dinda Susanti/Pradanna Putra Tampi/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679321/mendag-targetkan-neraca-dagang-pada-juli-2026-kembali-surplus</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
+      <c r="G79" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-160042.jpg</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
         <is>
           <t>TNI tembus medan ekstrem selama 12 hari antarkan bantuan ke Puncak</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
         <is>
           <t>ANTARA - Komando Operasi TNI Habema berhasil menyalurkan dua ton bantuan kemanusiaan kepada masyarakat di Distrik Agandugume, Oneri, dan Lambewi, Kabupaten Puncak, Papua Tengah. Bantuan tersebut tiba setelah personel TNI berjalan kaki  selama 12 hari melintasi pegunungan dengan medan ekstrem dan cuaca yang tidak menentu. (Laksa Mahendra/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679297/tni-tembus-medan-ekstrem-selama-12-hari-antarkan-bantuan-ke-puncak</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G80" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_TNI-TEMBUS-MEDAN-EKSTREM-SELAMA-12-HARI-ANTARKAN-BANTUAN-KE-PUNCAK.jpg</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
         <is>
           <t>Menko Zulhas bantah isu Kopdes penyebab tutupnya warung kelontong</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Koordinator Bidang Pangan, Zulkifli Hasan, membantah isu yang menyebut kehadiran Koperasi Desa/Kelurahan Merah Putih akan menyebabkan penutupan warung kelontong. Zulhas menegaskan Koperasi Merah Putih merupakan infrastruktur pemerintah yang dibentuk untuk memperkuat penyaluran berbagai subsidi dan bantuan kepada masyarakat. (Shintia Aryanti Krisna/Dudy Yanuwardhana/Winanto)</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F81" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679253/menko-zulhas-bantah-isu-kopdes-penyebab-tutupnya-warung-kelontong</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/MENKO-ZULHAS-BANTAH-ISU-KOPDES.jpg</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
         <is>
           <t>Pemkot Yogyakarta berikan vaksin HPV perdana pada anak laki-laki</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
         <is>
           <t>ANTARA -Dinas Kesehatan Kota Yogyakarta memperluas sasaran program Vaksinasi Human Papillomavirus (HPV) yang tidak hanya diperuntukan bagi anak perempuan, namun juga menyasar anak laki-laki usia 11 tahun. Pemberian vaksin HPV tersebut dilakukan perdana di Sekolah Dasar Intis School Kotagede pada Selasa (4/8).(Imam Prasetyo Nugroho/Rizky Bagus Dhermawan/Ludmila Yusufin Diah Nastiti)</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679247/pemkot-yogyakarta-berikan-vaksin-hpv-perdana-pada-anak-laki-laki</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/Screenshot-2026-08-04-154404.jpg</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
         <is>
           <t>Pemerintah targetkan perdagangan RI-Thailand tembus 20 miliar dolar AS</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
         <is>
           <t>ANTARA - Menteri Perdagangan Budi Santoso usai menghadiri Indonesia-Thailand Business Forum, di Jakarta, Selasa (4/8), menyatakan, pemerintah menargetkan nilai perdagangan Indonesia dan Thailand meningkat menjadi lebih dari 20 miliar dolar AS dari posisi saat ini sebesar 17,7 miliar dolar AS. Target tersebut akan diupayakan melalui peningkatan pertemuan bilateral untuk mengurangi hambatan perdagangan dan memperluas akses pasar kedua negara. (Nabila Athifa/Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Winanto)</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679237/pemerintah-targetkan-perdagangan-ri-thailand-tembus-20-miliar-dolar-as</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_PEMERINTAH-TARGETKAN-PERDAGANGAN-RI-THAILAND-TEMBUS-20-MILIAR-DOLAR-AS.jpg</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
         <is>
           <t>Pemkab Banjarnegara fasilitasi warga deteksi dini kesehatan mata</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
         <is>
           <t>ANTARA - Pemerintah Kabupaten Banjarnegara, Jawa Tengah, bersama Yayasan Satu Karsa Karya (YSKK) meluncurkan program penguatan sistem dan pelayanan kesehatan mata yang efektif dan inklusif. Kegiatan ini  merupakan upaya untuk mencegah gangguan penglihatan dan katarak dengan penanganan terintegrasi dari tingkat pelayanan primer hingga sekunder melalui penjaringan keluhan pada berbagai kelembagaan yang dekat dengan masyarakat. (Addin Alfath Amajida/Dudy Yanuwardhana/Winanto)</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679229/pemkab-banjarnegara-fasilitasi-warga-deteksi-dini-kesehatan-mata</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/PEMKAB-BANJARNEGARA-FASILITASI-WARGA.jpg</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>antara</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
         <is>
           <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Wed, 05 Aug 2026 05:10:02 +0700</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Wed, 05 Aug 2026 06:50:01 +0700</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
         <is>
           <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa (4/8), yang dihadiri Perdana Menteri (PM) Thailand Anutin Charnvirakul. Dalam kesempatan tersebut ditandatangani sejumlah perjanjian kerja sama di bidang perekonomian. (Sanya Dinda Susanti/Pradanna Putra Tampi/Andi Bagasela/Roy Rosa Bachtiar)</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
+      <c r="G85" t="inlineStr">
         <is>
           <t>https://img.antaranews.com/video/preview/2026/08/small/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H85" t="inlineStr">
         <is>
           <t>antara</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H77"/>
+  <autoFilter ref="A1:H85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>